<commit_message>
Qualys CI lookup rules V3.0: three rules for the unmatched population (management controllers, network interfaces, load balancer services)
281,700 unmatched Discovered Items profiled (stored-column aggregates plus a 4,800-row spread
sample); analysis workbook by evidence group. Rules 420, 430 and 460 added with six
usem.ci_lookup.* properties, generated in the same comment style; 18 cases run twice through
CIIdentify.identify (positive, negative, ambiguity, regression), all passing. Set V3.0 (Global,
9 updates) natively exported and proven through the upload path.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UaiSzs85tKmfaeLA1rAxsP
</commit_message>
<xml_diff>
--- a/stories/qualys-ci-lookup-rules/Qualys CI Lookup Rules - Code Line Explanations.xlsx
+++ b/stories/qualys-ci-lookup-rules/Qualys CI Lookup Rules - Code Line Explanations.xlsx
@@ -18,15 +18,18 @@
     <sheet name="350 Layered DNS Match" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="400 Hostname Class Match" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="410 Hostname Hardware Match" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="450 FQDN Name Hardware Match" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="700 IP Class Match" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="705 IP Hardware Match" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="730 IP Adapter Match" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="740 IP Layered Match" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="850 FQDN Name Broad Match" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="420 Management Interface Match" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="430 Network Interface Name Matc" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="450 FQDN Name Hardware Match" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="460 Load Balancer Service Match" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="700 IP Class Match" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="705 IP Hardware Match" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="730 IP Adapter Match" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="740 IP Layered Match" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="850 FQDN Name Broad Match" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overview'!$A$1:$I$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overview'!$A$1:$I$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1068,44 +1071,146 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>USEM Management Interface Match</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>DNS</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Match the management controller of a server (HP iLO, Oracle ILOM, Dell iDRAC, IBM IMM, Cisco CIMC, generic BMC or IPMI) to the server itself. Controllers are scanned under their own DNS label, which is the server name plus a suffix ("-ilo", "-ilom", "-idrac"), so the name rules never find them. The findings belong to the server owner.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>400/410 tried the full label "tx6dd630001-ilo" as a hostname and found nothing, because no CI is named after the controller.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>hosts whose label ends with a listed controller suffix, or whose OS text names a controller (property lists usem.ci_lookup.mgmt_suffixes and usem.ci_lookup.mgmt_os_markers).</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>430 (network interface names) and 450 (CI named with the full FQDN).</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>the hardware CI named "tx6dd630001" (the label without "-ilo"), for example a Linux Server; null when no CI or two CIs carry that name, or when the CI is a load balancer.</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "1201534877",
+  "IP": "159.185.200.11",
+  "TRACKING_METHOD": "IP",
+  "OS": "HP iLO",
+  "DNS": "tx6dd630001-ilo.bankofamerica.com"
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>430</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>USEM Network Interface Name Match</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>DNS</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Match a network device scanned through one of its interface or VLAN addresses. Such addresses carry a DNS label made of the device name plus an interface tail ("-cz04-hsrp-vlan705", "-atm1-v201", "-aom"), and the device CI is named by the leading part only. The rule walks the label from the longest prefix to the shortest and accepts the first prefix that names exactly one Network Gear CI.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>400/410 tried the whole label as a hostname; 420 looked for a management controller suffix.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>hosts whose DNS domain is an interface domain (".network." by default, property usem.ci_lookup.interface_domains) or whose label contains an interface marker segment such as "vlan705", "v201", "hsrp", "aom" (property usem.ci_lookup.interface_markers).</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>450 (CI named with the full FQDN) and 460 (load balancer services).</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>the network device named "uspaltwrr01drm0119" (an IP Switch, router, firewall or load balancer device); null when no prefix names a device or when a prefix names two.</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "1187423005",
+  "IP": "171.149.3.49",
+  "TRACKING_METHOD": "IP",
+  "OS": "Linux 2.6",
+  "DNS": "uspaltwrr01drm0119-cz04-hsrp-vlan705.network.bankofamerica.com"
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
         <v>450</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>USEM FQDN Name Hardware Match</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>DNS</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Match CIs whose name field holds the complete FQDN string, in the hardware tree. Some CMDB loads (typically the appliance domains ending in .rpg) name the CI with the whole FQDN, so a short-name search can never find them.</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>every rule so far compared the short hostname or the fqdn field.</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>CIs named with the full FQDN, which none of the earlier rules can see.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>700 and above (IP address rules) and finally 850, the only rule allowed to search the broad cmdb_ci table by name.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>the hardware CI whose name is exactly "lva40bneehcs01.ecomm.devicenp.rpg", when it is the only one.</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>{
   "ID": "71973166",
@@ -1118,46 +1223,97 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>460</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>USEM Load Balancer Service Match</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Match a virtual IP answered by a load balancer to the Load Balancer Service CI that models it. The hardware rules deliberately refuse the balancer device, because a VIP is not the balancer; this rule gives such hosts their proper CI instead of leaving them unmatched. It runs on the IP field so that VIPs without a DNS name are covered too.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>175 to 450 searched the hardware tree and declined: a VIP has no serial, its name is not a server name, and the address belongs to a load balancer device, which those rules refuse.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>hosts with VIP evidence: an OS text naming a load balancer product (property usem.ci_lookup.vip_os_markers) or a DNS label with a VIP marker segment such as "-vip", "vs1" (property usem.ci_lookup.vip_markers).</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>700 and above (IP address rules) for hosts that are not VIPs.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>the Load Balancer Service CI whose fqdn is "crisp-tx.bankofamerica.com" (or, failing that, whose name is the DNS name or its label, or whose ip_address is "171.203.142.26"); null without VIP evidence, without a service, or when two services carry the value.</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "1202267231",
+  "IP": "171.203.142.26",
+  "TRACKING_METHOD": "IP",
+  "OS": "F5 Big IP",
+  "DNS": "crisp-tx.bankofamerica.com"
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
         <v>700</v>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>USEM IP Class Match</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>IP</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Match by IP address, inside the class the OS implies. An address is the least trustworthy identifier (addresses move between machines and are shared by load balancers), so it is used only when the host has no serial and no usable name, and only when exactly one CI of the agreed class carries it.</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>all serial and name rules (175 to 450). The sample has no DNS name, so every name rule declined.</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>DNS-less hosts, typically ESXi management interfaces and appliances (89 of the 21,000 hosts in the reference extract).</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>705 searches the address across all hardware with extra safety checks; 730 and 740 resolve it through adapters and the layered IP records.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>the ESX Server CI whose ip_address is "30.162.178.21", for example "vsdnac22xsdi009"; a load balancer or a Windows CI with the same address is outside the class and cannot be picked.</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>{
   "ID": "83047621",
@@ -1168,46 +1324,46 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
+    <row r="17">
+      <c r="A17" s="2" t="n">
         <v>705</v>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>USEM IP Hardware Match</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>IP</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Match by IP address anywhere in the hardware tree, with two extra safety checks: the CI must not be a load balancer, and its class must not contradict the scanned OS.</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>700 required the address to belong to one CI of the OS-implied class.</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>DNS-less hosts whose CI is classed generically (Server) or whose OS gave no class.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>730 (address on a network adapter) and 740 (layered IP Address records).</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>the one hardware CI whose ip_address is "30.162.178.21", accepted when it is an ESX Server or generically classed; rejected when it is a Load Balancer or a CI of a contradicting class such as Windows Server.</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>{
   "ID": "83047621",
@@ -1218,46 +1374,46 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
+    <row r="18">
+      <c r="A18" s="2" t="n">
         <v>730</v>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>USEM IP Adapter Match</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>IP</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Match by an IP address recorded on a Network Adapter record rather than on the CI itself (multi-homed servers, discovery-populated CIs). The adapter leads to its owning CI.</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>700/705 looked for the address in the ip_address field of the CI record itself.</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>hosts whose address is stored on an adapter record only.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>740 (layered IP Address records) and then the last-resort name rule 850.</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>the CI that owns the adapter carrying "30.162.178.21", for example adapter "vmk0" of the ESX Server "vsdnac22xsdi009"; declined when adapters of two different CIs carry the address or the owner is a load balancer.</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>{
   "ID": "83047621",
@@ -1268,46 +1424,46 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
+    <row r="19">
+      <c r="A19" s="2" t="n">
         <v>740</v>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>USEM IP Layered Match</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>IP</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Match by IP address through the layered model that CMDB discovery maintains: an IP Address record belongs to a Network Adapter, and the adapter belongs to the CI.</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>730 looked for the address on Network Adapter records.</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>hosts whose address exists only as an IP Address record in the layered model.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>850, the last-resort broad name search; if that also declines, the out-of-box Qualys rules (860 and above) get their turn.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>the CI at the end of the chain IP Address "30.162.178.21" -&gt; adapter "vmk0" -&gt; ESX Server "vsdnac22xsdi009"; declined for several owners or a load balancer.</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>{
   "ID": "83047621",
@@ -1318,46 +1474,46 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
+    <row r="20">
+      <c r="A20" s="2" t="n">
         <v>850</v>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>USEM FQDN Name Broad Match</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>DNS</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>The single, deliberately late, broad fallback: a CI named with the full FQDN anywhere in the CI table, classes outside the hardware tree included (a virtual machine instance, another logical CI). Still requires a unique owner outside the ignored classes.</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>every hardware-scoped rule (175 to 740) has declined for this host.</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>the rare CI named with the full FQDN that lives outside the hardware tree.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>the out-of-box Qualys rules: 860 QUALYS HOST ID, 880 Cloud Resource Id, 900 FQDN, 920 NetBIOS, 940 DNS, and 950/960 IP which are inactive by default.</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>the one CI in any class whose name is "lva40bneehcs01.ecomm.devicenp.rpg", for example a Virtual Machine Instance; declined when the name is shared.</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="I20" s="3" t="inlineStr">
         <is>
           <t>{
   "ID": "71973166",
@@ -1371,7 +1527,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I17"/>
+  <autoFilter ref="A1:I20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2712,6 +2868,1417 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Explanation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>(function process(rule, sourceValue, sourcePayload) {</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Entry point. The framework calls process(rule, sourceValue, sourcePayload) once per scanned host and uses what it returns: a CI sys_id links the host, null hands the host to the next rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (!sourceValue)
+        return null;</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>nothing to look up -&gt; null = "no match from this rule"</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var full = ('' + sourceValue).trim().toLowerCase();</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>"tx6dd630001-ilo.bankofamerica.com"</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var label = full.split('.')[0];</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>"tx6dd630001-ilo"</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var dash = label.lastIndexOf('-');</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>11, position of the last hyphen</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (dash &lt; 1)
+        return null;</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>no hyphen -&gt; nothing to strip -&gt; decline</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var os = ('' + (sourcePayload.OS || '')).toLowerCase();</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>"hp ilo"</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var ignore = (typeof _ignoreClass != 'undefined' &amp;&amp; _ignoreClass) ?
+        ('' + _ignoreClass) : gs.getProperty('sn_sec_cmn.ignoreCIClass', '');</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>CI classes that must never be matched (placeholder and technical classes). Administrators keep the list in the property sn_sec_cmn.ignoreCIClass; the framework may pass the same list in as _ignoreClass.
+Result: ignore = "sn_sec_cmn_unmatched_ci,sn_vul_qualys_ci,cmdb_ci_unclassed_hardware,cmdb_ci_incomplete_ip,cmdb_ci_dns_name"</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    function list(name, fallback) {</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>list() reads a comma separated system property into a lower-cased list, falling back to the default shipped with the rule. Administrators tune the rule by editing the property, not the script.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        var parts = ('' + gs.getProperty(name, fallback)).split(',');</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        var out = [];</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        for (var i = 0; i &lt; parts.length; i++) {</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            var item = parts[i].trim().toLowerCase();</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            if (item)
+                out.push(item);</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        }</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        return out;</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    }</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr"/>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Stage 1: Recognise a management controller and derive the server name</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr"/>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>What: the segment after the last hyphen is compared with the suffix list; when it is listed, the server name is the label without it. Otherwise the OS text is compared with the controller markers; when one is found, the last segment is stripped whatever it is, because controllers are named after their server with a site-specific tail such as "-r".
+Why: the two pieces of evidence cover both naming habits seen in the scans: an explicit suffix with any OS, and a controller OS with an arbitrary tail. Without either the host is not a controller and the rule must not touch it.
+Sample: "tx6dd630001-ilo" -&gt; tail "ilo" is listed -&gt; base = "tx6dd630001". "crpchictx103-r" with OS "HP iLO" -&gt; tail "r" is not listed, but the OS names a controller -&gt; base = "crpchictx103". "usposwks0042-x" with OS "Windows 10" -&gt; neither -&gt; decline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var suffixes = list('usem.ci_lookup.mgmt_suffixes', 'ilo,ilom,idrac,drac,ipmi,bmc,oob,mgmt,imm,cimc,rmm,con');</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var markers = list('usem.ci_lookup.mgmt_os_markers', 'ilo,ilom,idrac,drac,remote access controller,imm,cimc,bmc,ipmi,lights out');</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr"/>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var tail = label.substring(dash + 1);</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>"ilo"</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var base = '';</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (suffixes.indexOf(tail) != -1)
+        base = label.substring(0, dash);</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>listed suffix -&gt; "tx6dd630001"</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    else
+        for (var i = 0; i &lt; markers.length; i++)
+            if (os.indexOf(markers[i]) != -1) {</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                base = label.substring(0, dash);</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>controller OS -&gt; strip the last segment</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                break;</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            }</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Result: base = "tx6dd630001" for the sample; "" when the host shows no controller evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (!base)
+        return null;</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr"/>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Stage 2: Search the hardware tree for the server name</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr"/>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>What: opens a search on cmdb_ci_hardware, keeps only CIs whose name equals the derived server name, and leaves out the ignored classes.
+Why: the controller can sit in front of a server, a storage node or a network device, so the whole hardware tree is searched; safety comes from the uniqueness check that follows.
+Sample: the search on cmdb_ci_hardware for name = "tx6dd630001" finds the Linux Server "tx6dd630001".</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var gr = new GlideRecord('cmdb_ci_hardware');</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Hardware and every class beneath it</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    gr.addQuery('name', base);</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (ignore)
+        gr.addQuery('sys_class_name', 'NOT IN', ignore);</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>When the ignore list is filled, exclude those classes from the search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr"/>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Stage 3: Decide: exactly one CI that is not a load balancer, or decline</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr"/>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>What: runs the search, accepts the CI only when it is the single one, and refuses a load balancer.
+Why: two CIs with the server name cannot be told apart from the controller label alone, and a load balancer answering on a management address is still not the scanned host.
+Sample: one CI -&gt; return "3f2a9c7e1b8d4a5f9e6c0d2b7a4f8e1c". No CI -&gt; null and rule 430 gets its turn. Two CIs named "crpchictx103" -&gt; null.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr"/>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    gr.query();</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Runs the search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr"/>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (!gr.next())
+        return null;</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>no CI carries the server name -&gt; decline</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr"/>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var match = gr.getUniqueValue();</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>The sys_id of the CI found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (gr.hasNext())
+        return null;</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>two CIs carry it -&gt; never guess</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr"/>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var lb = new GlideRecord('cmdb_ci_lb');</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Search on the Load Balancer class.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr"/>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (lb.isValid() &amp;&amp; lb.get(match))
+        return null;</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>a load balancer is never the host</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr"/>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    return match;</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Result: the framework links the vulnerable item to the server and stops evaluating later rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr"/>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>})(rule, sourceValue, sourcePayload);</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Runs the function immediately with the values the framework supplied.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Explanation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>(function process(rule, sourceValue, sourcePayload) {</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Entry point. The framework calls process(rule, sourceValue, sourcePayload) once per scanned host and uses what it returns: a CI sys_id links the host, null hands the host to the next rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (!sourceValue)
+        return null;</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>nothing to look up -&gt; null = "no match from this rule"</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var full = ('' + sourceValue).trim().toLowerCase();</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>"uspaltwrr01drm0119-cz04-hsrp-vlan705.network.bankofamerica.com"</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var label = full.split('.')[0];</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>"uspaltwrr01drm0119-cz04-hsrp-vlan705"</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var segments = label.split('-');</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>["uspaltwrr01drm0119", "cz04", "hsrp", "vlan705"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (segments.length &lt; 2)
+        return null;</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>no hyphen -&gt; no interface tail -&gt; decline</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var ignore = (typeof _ignoreClass != 'undefined' &amp;&amp; _ignoreClass) ?
+        ('' + _ignoreClass) : gs.getProperty('sn_sec_cmn.ignoreCIClass', '');</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>CI classes that must never be matched (placeholder and technical classes). Administrators keep the list in the property sn_sec_cmn.ignoreCIClass; the framework may pass the same list in as _ignoreClass.
+Result: ignore = "sn_sec_cmn_unmatched_ci,sn_vul_qualys_ci,cmdb_ci_unclassed_hardware,cmdb_ci_incomplete_ip,cmdb_ci_dns_name"</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    function list(name, fallback) {</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>list() reads a comma separated system property into a lower-cased list, falling back to the default shipped with the rule. Administrators tune the rule by editing the property, not the script.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        var parts = ('' + gs.getProperty(name, fallback)).split(',');</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        var out = [];</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        for (var i = 0; i &lt; parts.length; i++) {</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            var item = parts[i].trim().toLowerCase();</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            if (item)
+                out.push(item);</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        }</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        return out;</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    }</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    function isMarker(segment, words) {</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>isMarker() reports whether one hyphen segment of the label is a listed marker: the word itself ("vlan"), the word followed by digits only ("vlan705", "v201"), or, for words of three letters or more, a segment ending in the word ("multihostvip").</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        for (var i = 0; i &lt; words.length; i++) {</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            var w = words[i];</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            if (segment == w)
+                return true;</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr"/>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            if (segment.indexOf(w) == 0 &amp;&amp; /^[0-9]+$/.test(segment.substring(w.length)))
+                return true;</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            if (w.length &gt;= 3 &amp;&amp; segment.length &gt; w.length &amp;&amp; segment.substring(segment.length - w.length) == w)
+                return true;</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        }</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        return false;</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    }</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr"/>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Stage 1: Require interface evidence</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr"/>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>What: the rule goes on only when the DNS domain contains a listed interface domain, or one of the segments after the first is a listed interface marker.
+Why: plenty of ordinary server names contain hyphens ("ah-1047132-001"); without the interface evidence the prefix walk would strip real hostnames and could land on an unrelated device.
+Sample: ".network." is found in the sample name -&gt; evidence. "gtcmmrlpa05a-vlan10.corp.bankofamerica.com" -&gt; segment "vlan10" is a marker -&gt; evidence. "ah-1047132-001.corp.bankofamerica.com" -&gt; neither -&gt; decline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var domains = list('usem.ci_lookup.interface_domains', '.network.');</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var markers = list('usem.ci_lookup.interface_markers', 'vlan,v,hsrp,vrrp,po,eth,gi,te,lo,mgmt,aom,vs,fab');</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var evidence = false;</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    for (var d = 0; d &lt; domains.length; d++)
+        if (full.indexOf(domains[d]) != -1)
+            evidence = true;</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    for (var s = 1; s &lt; segments.length; s++)
+        if (isMarker(segments[s], markers))
+            evidence = true;</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Result: evidence = true for the sample (the domain contains ".network." and "vlan705" is a marker)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (!evidence)
+        return null;</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr"/>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Stage 2: Walk the prefixes from the longest to the shortest against Network Gear</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr"/>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>What: drops one segment at a time from the right and searches Network Gear (switches, routers, firewalls) and Load Balancer devices for a CI with exactly that name. The first prefix that finds anything decides: one CI is the match, two CIs mean the rule declines.
+Why: the device name is the leading part of the label but its length varies by site; trying the longest prefix first keeps "site-device-01" from being cut down to "site" when a CI named with the longer form exists.
+Sample: prefixes tried: "uspaltwrr01drm0119-cz04-hsrp" (none), "uspaltwrr01drm0119-cz04" (none), "uspaltwrr01drm0119" (the IP Switch "uspaltwrr01drm0119") -&gt; return "3f2a9c7e1b8d4a5f9e6c0d2b7a4f8e1c". Two switches named "ustxrdnwl01rsm004z" -&gt; null.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr"/>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var tables = ['cmdb_ci_netgear', 'cmdb_ci_lb'];</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Network devices live in two branches of the CMDB: Network Gear (switches, routers, firewalls) and Load Balancer, which the platform files under Server. Both are searched; the hits are counted together.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr"/>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    for (var k = segments.length - 1; k &gt;= 1; k--) {</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr"/>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        var base = segments.slice(0, k).join('-');</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>"uspaltwrr01drm0119-cz04-hsrp", then "uspaltwrr01drm0119-cz04", then "uspaltwrr01drm0119"</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        var hits = [];</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>sys_ids of the devices named exactly like this prefix</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr"/>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        for (var t = 0; t &lt; tables.length; t++) {</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr"/>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            var gr = new GlideRecord(tables[t]);</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr"/>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            if (!gr.isValid())
+                continue;</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>The class is not installed on this instance -&gt; decline rather than fail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr"/>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            gr.addQuery('name', base);</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr"/>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            if (ignore)
+                gr.addQuery('sys_class_name', 'NOT IN', ignore);</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>When the ignore list is filled, exclude those classes from the search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr"/>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            gr.query();</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Runs the search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr"/>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            while (gr.next() &amp;&amp; hits.length &lt; 2)
+                hits.push(gr.getUniqueValue());</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr"/>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        }</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr"/>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        if (hits.length == 0)
+            continue;</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>nothing named like this -&gt; try a shorter prefix</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr"/>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        if (hits.length &gt; 1)
+            return null;</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>two devices carry this name -&gt; never guess</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr"/>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        return hits[0];</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr"/>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    }</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr"/>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    return null;</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Result: no prefix names a device -&gt; decline; the host continues to rule 450</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr"/>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>})(rule, sourceValue, sourcePayload);</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Runs the function immediately with the values the framework supplied.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3011,7 +4578,829 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Explanation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>(function process(rule, sourceValue, sourcePayload) {</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Entry point. The framework calls process(rule, sourceValue, sourcePayload) once per scanned host and uses what it returns: a CI sys_id links the host, null hands the host to the next rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (!sourceValue)
+        return null;</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>nothing to look up -&gt; null = "no match from this rule"</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var ip = ('' + sourceValue).trim();</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>"171.203.142.26"</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (!ip || ip.indexOf('127.') == 0 || ip.indexOf('169.254.') == 0)
+        return null;</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>loopback and link-local identify nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var dns = ('' + (sourcePayload.DNS || '')).trim().toLowerCase();</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>"crisp-tx.bankofamerica.com" or ""</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var label = dns.split('.')[0];</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>"crisp-tx"</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var os = ('' + (sourcePayload.OS || '')).toLowerCase();</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>"f5 big ip"</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var ignore = (typeof _ignoreClass != 'undefined' &amp;&amp; _ignoreClass) ?
+        ('' + _ignoreClass) : gs.getProperty('sn_sec_cmn.ignoreCIClass', '');</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>CI classes that must never be matched (placeholder and technical classes). Administrators keep the list in the property sn_sec_cmn.ignoreCIClass; the framework may pass the same list in as _ignoreClass.
+Result: ignore = "sn_sec_cmn_unmatched_ci,sn_vul_qualys_ci,cmdb_ci_unclassed_hardware,cmdb_ci_incomplete_ip,cmdb_ci_dns_name"</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    function list(name, fallback) {</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>list() reads a comma separated system property into a lower-cased list, falling back to the default shipped with the rule. Administrators tune the rule by editing the property, not the script.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        var parts = ('' + gs.getProperty(name, fallback)).split(',');</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        var out = [];</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        for (var i = 0; i &lt; parts.length; i++) {</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            var item = parts[i].trim().toLowerCase();</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            if (item)
+                out.push(item);</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        }</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        return out;</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    }</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    function isMarker(segment, words) {</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>isMarker() reports whether one hyphen segment of the label is a listed marker: the word itself ("vlan"), the word followed by digits only ("vlan705", "v201"), or, for words of three letters or more, a segment ending in the word ("multihostvip").</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        for (var i = 0; i &lt; words.length; i++) {</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            var w = words[i];</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr"/>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            if (segment == w)
+                return true;</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            if (segment.indexOf(w) == 0 &amp;&amp; /^[0-9]+$/.test(segment.substring(w.length)))
+                return true;</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            if (w.length &gt;= 3 &amp;&amp; segment.length &gt; w.length &amp;&amp; segment.substring(segment.length - w.length) == w)
+                return true;</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        }</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        return false;</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    }</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr"/>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Stage 1: Require VIP evidence</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr"/>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>What: the rule goes on only when the OS text contains a listed load balancer product word, or one of the label segments is a listed VIP marker.
+Why: a Load Balancer Service must never be returned for an ordinary server that happens to share an address with a VIP; the evidence keeps this rule to the hosts that really are VIPs.
+Sample: "f5 big ip" contains "f5" -&gt; evidence. "rbps-dev3-sve-vip.ecommnp.rpg" with OS "Linux 2.6" -&gt; segment "vip" -&gt; evidence. "ah-1047132-001" with OS "Red Hat Enterprise Linux 9.8" -&gt; neither -&gt; decline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var osMarkers = list('usem.ci_lookup.vip_os_markers', 'f5,big-ip,big ip,netscaler');</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var labelMarkers = list('usem.ci_lookup.vip_markers', 'vip,vs');</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var evidence = false;</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    for (var m = 0; m &lt; osMarkers.length; m++)
+        if (os.indexOf(osMarkers[m]) != -1)
+            evidence = true;</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var segments = label ? label.split('-') : [];</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr"/>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    for (var s = 0; s &lt; segments.length; s++)
+        if (isMarker(segments[s], labelMarkers))
+            evidence = true;</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Result: evidence = true for the sample</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr"/>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (!evidence)
+        return null;</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr"/>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Stage 2: Find the one Load Balancer Service by fqdn, then by name, then by address</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr"/>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>What: searches cmdb_ci_lb_service (and its sub-classes) for the scanned DNS name in the fqdn field, then in the name field, then for the label in the name field, then for the scanned address in ip_address. Each step accepts exactly one service; a step that finds two services ends the rule with null, a step that finds nothing hands over to the next step.
+Why: the most specific evidence is tried first, and an ambiguous answer is never skipped over to a weaker one, because the weaker evidence could pick a different service.
+Sample: fqdn = "crisp-tx.bankofamerica.com" finds the Load Balancer Service "crisp-tx" -&gt; return "3f2a9c7e1b8d4a5f9e6c0d2b7a4f8e1c". A VIP with two services on the same address and no DNS -&gt; null.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr"/>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    function one(field, value) {</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        if (!value)
+            return undefined;</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>no value to search -&gt; next step</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr"/>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        var gr = new GlideRecord('cmdb_ci_lb_service');</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr"/>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        if (!gr.isValid())
+            return null;</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>class not installed -&gt; decline</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr"/>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        gr.addQuery(field, value);</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr"/>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        if (ignore)
+            gr.addQuery('sys_class_name', 'NOT IN', ignore);</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>When the ignore list is filled, exclude those classes from the search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr"/>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        gr.query();</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Runs the search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr"/>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        if (!gr.next())
+            return undefined;</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>nothing found -&gt; next step</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr"/>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        var id = gr.getUniqueValue();</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>The sys_id of the CI found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr"/>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        if (gr.hasNext())
+            return null;</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>two services -&gt; never guess</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr"/>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        return id;</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>The CI passed every check -&gt; its sys_id goes back to the framework.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr"/>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    }</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr"/>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var steps = [['fqdn', dns], ['name', dns], ['name', label], ['ip_address', ip]];</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr"/>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    for (var t = 0; t &lt; steps.length; t++) {</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr"/>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        var found = one(steps[t][0], steps[t][1]);</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr"/>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        if (found === null)
+            return null;</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>ambiguous at this step -&gt; decline</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr"/>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        if (found)
+            return found;</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>exactly one service -&gt; match</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr"/>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    }</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr"/>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    return null;</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Result: no service for any of the evidence -&gt; decline; the host continues to rule 700</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr"/>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>})(rule, sourceValue, sourcePayload);</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Runs the function immediately with the values the framework supplied.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3622,7 +6011,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4402,7 +6791,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4903,7 +7292,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5411,311 +7800,6 @@
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>Runs the function immediately with the values the framework supplied.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Stage</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Explanation</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>(function process(rule, sourceValue, sourcePayload) {</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Entry point. The framework calls process(rule, sourceValue, sourcePayload) once per scanned host and uses what it returns: a CI sys_id links the host, null hands the host to the next rule.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr"/>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    if (!sourceValue)
-        return null;</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>nothing to look up -&gt; null = "no match from this rule"</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    var fqdn = ('' + sourceValue).trim().toLowerCase();</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>"lva40bneehcs01.ecomm.devicenp.rpg"</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr"/>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    if (fqdn.indexOf('.') == -1)
-        return null;</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>no domain part -&gt; the hostname rules (400+) handle bare labels</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    var ignore = (typeof _ignoreClass != 'undefined' &amp;&amp; _ignoreClass) ?
-        ('' + _ignoreClass) : gs.getProperty('sn_sec_cmn.ignoreCIClass', '');</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>CI classes that must never be matched (placeholder and technical classes). Administrators keep the list in the property sn_sec_cmn.ignoreCIClass; the framework may pass the same list in as _ignoreClass.
-Result: ignore = "sn_sec_cmn_unmatched_ci,sn_vul_qualys_ci,cmdb_ci_unclassed_hardware,cmdb_ci_incomplete_ip,cmdb_ci_dns_name"</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr"/>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Stage 1: Search the whole CI table for a CI named with the full FQDN</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr"/>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>What: opens a search on cmdb_ci, the root of every CI class, keeps only CIs whose name equals the complete lower-cased DNS name, and leaves out the ignored classes.
-Why: this is the only USEM rule that searches outside the hardware tree, which is why it runs last: every more precise rule has had its chance, and the ignore list still keeps placeholder classes out.
-Sample: the search on cmdb_ci for name = "lva40bneehcs01.ecomm.devicenp.rpg" finds the Virtual Machine Instance "lva40bneehcs01.ecomm.devicenp.rpg".</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    var gr = new GlideRecord('cmdb_ci');</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>the root CI table, every class</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr"/>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    gr.addQuery('name', fqdn);</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Condition: name equals the complete DNS name.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" s="2" t="inlineStr"/>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    if (ignore)
-        gr.addQuery('sys_class_name', 'NOT IN', ignore);</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>When the ignore list is filled, exclude those classes from the search.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr"/>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Stage 2: Decide: exactly one CI, or decline</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr"/>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>What: runs the search, reads the first CI and accepts it only when no second CI is in the result.
-Why: every finding of this host is linked to the CI returned; a wrong CI sends findings to the wrong owner. Two CIs sharing the value is an ambiguity, so the rule declines and a later rule with different evidence may still resolve the host.
-Sample: one CI (the Virtual Machine Instance "lva40bneehcs01.ecomm.devicenp.rpg") -&gt; return "3f2a9c7e1b8d4a5f9e6c0d2b7a4f8e1c". No CI -&gt; return null; the out-of-box Qualys rules (860 and above) get their turn. Two CIs -&gt; two CIs with that full name -&gt; return null.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="2" t="inlineStr"/>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    gr.query();</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Runs the search.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B13" s="2" t="inlineStr"/>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    if (!gr.next())
-        return null;</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>empty result -&gt; decline</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B14" s="2" t="inlineStr"/>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    var match = gr.getUniqueValue();</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Result: match = "3f2a9c7e1b8d4a5f9e6c0d2b7a4f8e1c", the sys_id of the Virtual Machine Instance "lva40bneehcs01.ecomm.devicenp.rpg"</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B15" s="2" t="inlineStr"/>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    if (gr.hasNext())
-        return null;</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>a second CI carries the same value -&gt; never guess</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B16" s="2" t="inlineStr"/>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    return match;</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Result: the framework links the vulnerable item to this CI and stops evaluating later rules</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="B17" s="2" t="inlineStr"/>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>})(rule, sourceValue, sourcePayload);</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Runs the function immediately with the values the framework supplied.</t>
         </is>
@@ -6355,6 +8439,311 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Explanation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>(function process(rule, sourceValue, sourcePayload) {</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Entry point. The framework calls process(rule, sourceValue, sourcePayload) once per scanned host and uses what it returns: a CI sys_id links the host, null hands the host to the next rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (!sourceValue)
+        return null;</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>nothing to look up -&gt; null = "no match from this rule"</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var fqdn = ('' + sourceValue).trim().toLowerCase();</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>"lva40bneehcs01.ecomm.devicenp.rpg"</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (fqdn.indexOf('.') == -1)
+        return null;</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>no domain part -&gt; the hostname rules (400+) handle bare labels</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var ignore = (typeof _ignoreClass != 'undefined' &amp;&amp; _ignoreClass) ?
+        ('' + _ignoreClass) : gs.getProperty('sn_sec_cmn.ignoreCIClass', '');</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>CI classes that must never be matched (placeholder and technical classes). Administrators keep the list in the property sn_sec_cmn.ignoreCIClass; the framework may pass the same list in as _ignoreClass.
+Result: ignore = "sn_sec_cmn_unmatched_ci,sn_vul_qualys_ci,cmdb_ci_unclassed_hardware,cmdb_ci_incomplete_ip,cmdb_ci_dns_name"</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr"/>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Stage 1: Search the whole CI table for a CI named with the full FQDN</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr"/>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>What: opens a search on cmdb_ci, the root of every CI class, keeps only CIs whose name equals the complete lower-cased DNS name, and leaves out the ignored classes.
+Why: this is the only USEM rule that searches outside the hardware tree, which is why it runs last: every more precise rule has had its chance, and the ignore list still keeps placeholder classes out.
+Sample: the search on cmdb_ci for name = "lva40bneehcs01.ecomm.devicenp.rpg" finds the Virtual Machine Instance "lva40bneehcs01.ecomm.devicenp.rpg".</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var gr = new GlideRecord('cmdb_ci');</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>the root CI table, every class</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    gr.addQuery('name', fqdn);</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Condition: name equals the complete DNS name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (ignore)
+        gr.addQuery('sys_class_name', 'NOT IN', ignore);</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>When the ignore list is filled, exclude those classes from the search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Stage 2: Decide: exactly one CI, or decline</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr"/>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>What: runs the search, reads the first CI and accepts it only when no second CI is in the result.
+Why: every finding of this host is linked to the CI returned; a wrong CI sends findings to the wrong owner. Two CIs sharing the value is an ambiguity, so the rule declines and a later rule with different evidence may still resolve the host.
+Sample: one CI (the Virtual Machine Instance "lva40bneehcs01.ecomm.devicenp.rpg") -&gt; return "3f2a9c7e1b8d4a5f9e6c0d2b7a4f8e1c". No CI -&gt; return null; the out-of-box Qualys rules (860 and above) get their turn. Two CIs -&gt; two CIs with that full name -&gt; return null.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    gr.query();</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Runs the search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (!gr.next())
+        return null;</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>empty result -&gt; decline</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var match = gr.getUniqueValue();</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Result: match = "3f2a9c7e1b8d4a5f9e6c0d2b7a4f8e1c", the sys_id of the Virtual Machine Instance "lva40bneehcs01.ecomm.devicenp.rpg"</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (gr.hasNext())
+        return null;</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>a second CI carries the same value -&gt; never guess</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    return match;</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Result: the framework links the vulnerable item to this CI and stops evaluating later rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>})(rule, sourceValue, sourcePayload);</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Runs the function immediately with the values the framework supplied.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Qualys CI lookup rules V3.2: lists inline in rules 420/430/460, no custom properties; deck and workbook aligned
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UaiSzs85tKmfaeLA1rAxsP
</commit_message>
<xml_diff>
--- a/stories/qualys-ci-lookup-rules/Qualys CI Lookup Rules - Code Line Explanations.xlsx
+++ b/stories/qualys-ci-lookup-rules/Qualys CI Lookup Rules - Code Line Explanations.xlsx
@@ -1,32 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="175 Serial Number Class Match" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="180 Serial Number Hardware Matc" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="200 Cisco IP Phone MAC" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="250 FQDN Class Match" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="260 FQDN Hardware Match" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="300 Hostname Domain Class Match" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="310 Hostname Domain Hardware Ma" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="350 Layered DNS Match" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="400 Hostname Class Match" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="410 Hostname Hardware Match" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="420 Management Interface Match" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="430 Network Interface Name Matc" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="450 FQDN Name Hardware Match" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="460 Load Balancer Service Match" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="700 IP Class Match" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="705 IP Hardware Match" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="730 IP Adapter Match" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="740 IP Layered Match" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="850 FQDN Name Broad Match" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="175 Serial Number Class Match" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="180 Serial Number Hardware Matc" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="200 Cisco IP Phone MAC" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="250 FQDN Class Match" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="260 FQDN Hardware Match" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="300 Hostname Domain Class Match" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="310 Hostname Domain Hardware Ma" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="350 Layered DNS Match" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="400 Hostname Class Match" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="410 Hostname Hardware Match" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="420 Management Interface Match" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="430 Network Interface Name Matc" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="450 FQDN Name Hardware Match" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="460 Load Balancer Service Match" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="700 IP Class Match" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="705 IP Hardware Match" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="730 IP Adapter Match" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="740 IP Layered Match" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="850 FQDN Name Broad Match" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overview'!$A$1:$I$20</definedName>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>hosts whose label ends with a listed controller suffix, or whose OS text names a controller (properties usem.ci_lookup.mgmt_suffixes and usem.ci_lookup.mgmt_os_markers).</t>
+          <t>hosts whose label ends with one of the controller suffixes, or whose OS text names a controller; both lists are declared in the script, at the top of the matching stage.</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>hosts whose DNS domain is an interface domain (".network." in our feed, property usem.ci_lookup.interface_domains) or whose label contains an interface marker segment such as "vlan705", "v201", "hsrp", "aom" (property usem.ci_lookup.interface_markers).</t>
+          <t>hosts whose DNS domain is an interface domain (".network." in our feed) or whose label contains an interface marker segment such as "vlan705", "v201", "hsrp", "aom"; both lists are declared in the script, at the top of the matching stage.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>hosts with VIP evidence: an OS text naming a load balancer product (property usem.ci_lookup.vip_os_markers) or a DNS label with a VIP marker segment such as "-vip" or "vs1" (property usem.ci_lookup.vip_markers).</t>
+          <t>hosts with VIP evidence: an OS text naming a load balancer product, or a DNS label with a VIP marker segment such as "-vip" or "vs1"; both lists are declared in the script, at the top of the matching stage.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -2732,7 +2732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2895,161 +2895,163 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="inlineStr"/>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    function list(name, fallback) {</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>list() reads a comma separated system property into a lower-cased list, falling back to the default shipped with the rule; the lists are tuned in the properties, not in the script.</t>
+      <c r="A10" s="4" t="inlineStr"/>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Recognise a controller and derive the server name</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>The segment after the last hyphen is checked against the suffix list; when it is listed the server name is the label without it. Otherwise the OS text is checked for a controller word, and then the last segment is stripped whatever it is, because some controllers carry a site-specific tail instead ("crpchictx103-r" with OS "HP iLO"). Both habits are in the feed. Without either piece of evidence the host is not a controller and the rule must not touch it ("usposwks0042-x" with a Windows OS stays with the name rules). The label suffixes that mark a controller, and the words that name one in the OS text. Extend these two lists when a site uses another naming habit.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" s="2" t="inlineStr"/>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        var parts = ('' + gs.getProperty(name, fallback)).split(',');</t>
+          <t xml:space="preserve">    var suffixes = ['ilo', 'ilom', 'idrac', 'drac', 'ipmi', 'bmc', 'oob', 'mgmt', 'imm', 'cimc', 'rmm', 'con'];</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Read the property (or the default shipped with the rule) and split it on commas.</t>
+          <t>The label suffixes that mark a management controller.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" s="2" t="inlineStr"/>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        var out = [];</t>
+          <t xml:space="preserve">    var markers = ['ilo', 'ilom', 'idrac', 'drac', 'remote access controller', 'imm', 'cimc', 'bmc', 'ipmi', 'lights out'];</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>The cleaned list.</t>
+          <t>The words that name a controller in the OS text.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" s="2" t="inlineStr"/>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        for (var i = 0; i &lt; parts.length; i++) {</t>
+          <t xml:space="preserve">    var tail = label.substring(dash + 1);</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Loop over the comma separated entries.</t>
+          <t>"ilo"</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" s="2" t="inlineStr"/>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">            var item = parts[i].trim().toLowerCase();</t>
+          <t xml:space="preserve">    var base = '';</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Trim and lower-case one entry.</t>
+          <t>The server name once derived; stays empty without controller evidence.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" s="2" t="inlineStr"/>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">            if (item)
-                out.push(item);</t>
+          <t xml:space="preserve">    if (suffixes.indexOf(tail) != -1)
+        base = label.substring(0, dash);</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Keep non-empty entries.</t>
+          <t>listed suffix: "tx6dd630001"</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" s="2" t="inlineStr"/>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        }</t>
+          <t xml:space="preserve">    else
+        for (var i = 0; i &lt; markers.length; i++)
+            if (os.indexOf(markers[i]) != -1) {</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>End of the block.</t>
+          <t>No listed suffix: when the OS text names a controller, strip the last segment whatever it is.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17" s="2" t="inlineStr"/>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        return out;</t>
+          <t xml:space="preserve">                base = label.substring(0, dash);</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>The list of lower-cased entries.</t>
+          <t>controller OS: strip the last segment</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B18" s="2" t="inlineStr"/>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    }</t>
+          <t xml:space="preserve">                break;</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
+          <t>One controller word is enough.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            }</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
           <t>End of the block.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr"/>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Recognise a controller and derive the server name</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr"/>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>The segment after the last hyphen is checked against the suffix list; when it is listed the server name is the label without it. Otherwise the OS text is checked for a controller word, and then the last segment is stripped whatever it is, because some controllers carry a site-specific tail instead ("crpchictx103-r" with OS "HP iLO"). Both habits are in the feed. Without either piece of evidence the host is not a controller and the rule must not touch it ("usposwks0042-x" with a Windows OS stays with the name rules).</t>
         </is>
       </c>
     </row>
@@ -3060,174 +3062,175 @@
       <c r="B20" s="2" t="inlineStr"/>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    var suffixes = list('usem.ci_lookup.mgmt_suffixes', 'ilo,ilom,idrac,drac,ipmi,bmc,oob,mgmt,imm,cimc,rmm,con');</t>
+          <t xml:space="preserve">    if (!base)
+        return null;</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Controller suffixes, from the property (defaults shipped with the rule).</t>
+          <t>No controller evidence -&gt; decline untouched.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="B21" s="2" t="inlineStr"/>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    var markers = list('usem.ci_lookup.mgmt_os_markers', 'ilo,ilom,idrac,drac,remote access controller,imm,cimc,bmc,ipmi,lights out');</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Controller words looked for in the OS text, from the property.</t>
+      <c r="A21" s="4" t="inlineStr"/>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>The server by name, across the hardware tree, one CI only</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr"/>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>The controller can sit in front of a server, a storage node or a network device, so the whole hardware tree is searched. Two CIs with the server name cannot be told apart from the controller label alone and the rule declines; a load balancer is refused because a balancer answering on a management address is still not the scanned host.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B22" s="2" t="inlineStr"/>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    var tail = label.substring(dash + 1);</t>
+          <t xml:space="preserve">    var gr = new GlideRecord('cmdb_ci_hardware');</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>"ilo"</t>
+          <t>Hardware and every class beneath it</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B23" s="2" t="inlineStr"/>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    var base = '';</t>
+          <t xml:space="preserve">    gr.addQuery('name', base);</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>The server name once derived; stays empty without controller evidence.</t>
+          <t>Condition: name equals the derived name.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B24" s="2" t="inlineStr"/>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    if (suffixes.indexOf(tail) != -1)
-        base = label.substring(0, dash);</t>
+          <t xml:space="preserve">    if (ignore)
+        gr.addQuery('sys_class_name', 'NOT IN', ignore);</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>listed suffix: "tx6dd630001"</t>
+          <t>When the ignore list is filled, exclude those classes from the search.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B25" s="2" t="inlineStr"/>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    else
-        for (var i = 0; i &lt; markers.length; i++)
-            if (os.indexOf(markers[i]) != -1) {</t>
+          <t xml:space="preserve">    gr.query();</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>No listed suffix: when the OS text names a controller, strip the last segment whatever it is.</t>
+          <t>Runs the search.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B26" s="2" t="inlineStr"/>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                base = label.substring(0, dash);</t>
+          <t xml:space="preserve">    if (!gr.next())
+        return null;</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>controller OS: strip the last segment</t>
+          <t>No row at all -&gt; decline.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B27" s="2" t="inlineStr"/>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                break;</t>
+          <t xml:space="preserve">    var match = gr.getUniqueValue();</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>One controller word is enough.</t>
+          <t>The sys_id of the CI found.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B28" s="2" t="inlineStr"/>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">            }</t>
+          <t xml:space="preserve">    if (gr.hasNext())
+        return null;</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>End of the block.</t>
+          <t>A second row means the value is shared by two CIs -&gt; decline rather than guess.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B29" s="2" t="inlineStr"/>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    if (!base)
+          <t xml:space="preserve">    var lb = new GlideRecord('cmdb_ci_lb');</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Search on the Load Balancer class.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (lb.isValid() &amp;&amp; lb.get(match))
         return null;</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>No controller evidence -&gt; decline untouched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr"/>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>The server by name, across the hardware tree, one CI only</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr"/>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>The controller can sit in front of a server, a storage node or a network device, so the whole hardware tree is searched. Two CIs with the server name cannot be told apart from the controller label alone and the rule declines; a load balancer is refused because a balancer answering on a management address is still not the scanned host.</t>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>The CI found is a load balancer -&gt; refuse it.</t>
         </is>
       </c>
     </row>
@@ -3238,12 +3241,12 @@
       <c r="B31" s="2" t="inlineStr"/>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    var gr = new GlideRecord('cmdb_ci_hardware');</t>
+          <t xml:space="preserve">    return match;</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Hardware and every class beneath it</t>
+          <t>Exactly one CI -&gt; return its sys_id; the framework links the host to it and stops the chain.</t>
         </is>
       </c>
     </row>
@@ -3254,158 +3257,10 @@
       <c r="B32" s="2" t="inlineStr"/>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    gr.addQuery('name', base);</t>
+          <t>})(rule, sourceValue, sourcePayload);</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Condition: name equals the derived name.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="B33" s="2" t="inlineStr"/>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    if (ignore)
-        gr.addQuery('sys_class_name', 'NOT IN', ignore);</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>When the ignore list is filled, exclude those classes from the search.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="B34" s="2" t="inlineStr"/>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    gr.query();</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Runs the search.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="B35" s="2" t="inlineStr"/>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    if (!gr.next())
-        return null;</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>No row at all -&gt; decline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="B36" s="2" t="inlineStr"/>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    var match = gr.getUniqueValue();</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>The sys_id of the CI found.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="B37" s="2" t="inlineStr"/>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    if (gr.hasNext())
-        return null;</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>A second row means the value is shared by two CIs -&gt; decline rather than guess.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="B38" s="2" t="inlineStr"/>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    var lb = new GlideRecord('cmdb_ci_lb');</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>Search on the Load Balancer class.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="n">
-        <v>36</v>
-      </c>
-      <c r="B39" s="2" t="inlineStr"/>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    if (lb.isValid() &amp;&amp; lb.get(match))
-        return null;</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>The CI found is a load balancer -&gt; refuse it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="B40" s="2" t="inlineStr"/>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    return match;</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>Exactly one CI -&gt; return its sys_id; the framework links the host to it and stops the chain.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="B41" s="2" t="inlineStr"/>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>})(rule, sourceValue, sourcePayload);</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>Runs the function immediately with the values the framework supplied.</t>
         </is>
@@ -3422,7 +3277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3575,12 +3430,12 @@
       <c r="B9" s="2" t="inlineStr"/>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    function list(name, fallback) {</t>
+          <t xml:space="preserve">    function isMarker(segment, words) {</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>list() reads a comma separated system property into a lower-cased list, falling back to the default shipped with the rule; the lists are tuned in the properties, not in the script.</t>
+          <t>isMarker() says whether one hyphen segment of the label is a listed marker: the word itself ("vlan"), the word followed by digits only ("vlan705", "v201"), or, for words of three letters or more, a segment ending in the word ("multihostvip").</t>
         </is>
       </c>
     </row>
@@ -3591,12 +3446,12 @@
       <c r="B10" s="2" t="inlineStr"/>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        var parts = ('' + gs.getProperty(name, fallback)).split(',');</t>
+          <t xml:space="preserve">        for (var i = 0; i &lt; words.length; i++) {</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Read the property (or the default shipped with the rule) and split it on commas.</t>
+          <t>Loop over the listed marker words.</t>
         </is>
       </c>
     </row>
@@ -3607,12 +3462,12 @@
       <c r="B11" s="2" t="inlineStr"/>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        var out = [];</t>
+          <t xml:space="preserve">            var w = words[i];</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>The cleaned list.</t>
+          <t>One marker word.</t>
         </is>
       </c>
     </row>
@@ -3623,12 +3478,13 @@
       <c r="B12" s="2" t="inlineStr"/>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        for (var i = 0; i &lt; parts.length; i++) {</t>
+          <t xml:space="preserve">            if (segment == w)
+                return true;</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Loop over the comma separated entries.</t>
+          <t>The segment is the word itself ("vlan").</t>
         </is>
       </c>
     </row>
@@ -3639,12 +3495,13 @@
       <c r="B13" s="2" t="inlineStr"/>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">            var item = parts[i].trim().toLowerCase();</t>
+          <t xml:space="preserve">            if (segment.indexOf(w) == 0 &amp;&amp; /^[0-9]+$/.test(segment.substring(w.length)))
+                return true;</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Trim and lower-case one entry.</t>
+          <t>The segment is the word followed by digits only ("vlan705", "v201").</t>
         </is>
       </c>
     </row>
@@ -3655,13 +3512,13 @@
       <c r="B14" s="2" t="inlineStr"/>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">            if (item)
-                out.push(item);</t>
+          <t xml:space="preserve">            if (w.length &gt;= 3 &amp;&amp; segment.length &gt; w.length &amp;&amp; segment.substring(segment.length - w.length) == w)
+                return true;</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Keep non-empty entries.</t>
+          <t>For words of three letters or more, the segment ends in the word ("multihostvip").</t>
         </is>
       </c>
     </row>
@@ -3688,12 +3545,12 @@
       <c r="B16" s="2" t="inlineStr"/>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        return out;</t>
+          <t xml:space="preserve">        return false;</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>The list of lower-cased entries.</t>
+          <t>No marker word fits this segment.</t>
         </is>
       </c>
     </row>
@@ -3714,278 +3571,277 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="2" t="inlineStr"/>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    function isMarker(segment, words) {</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>isMarker() says whether one hyphen segment of the label is a listed marker: the word itself ("vlan"), the word followed by digits only ("vlan705", "v201"), or, for words of three letters or more, a segment ending in the word ("multihostvip").</t>
+      <c r="A18" s="4" t="inlineStr"/>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Interface evidence first</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr"/>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>The rule goes on only when the DNS domain contains a listed interface domain or one of the segments after the first is a listed marker. Plenty of ordinary server names contain hyphens ("ah-1047132-001"); without this check the prefix walk would strip real hostnames and could land on an unrelated device. The domains under which devices are scanned per interface, and the label segments that mark an interface or VLAN address. Extend these two lists when a site uses another naming habit.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B19" s="2" t="inlineStr"/>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        for (var i = 0; i &lt; words.length; i++) {</t>
+          <t xml:space="preserve">    var domains = ['.network.'];</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Loop over the listed marker words.</t>
+          <t>The domains under which network devices are scanned per interface.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" s="2" t="inlineStr"/>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">            var w = words[i];</t>
+          <t xml:space="preserve">    var markers = ['vlan', 'v', 'hsrp', 'vrrp', 'po', 'eth', 'gi', 'te', 'lo', 'mgmt', 'aom', 'vs', 'fab'];</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>One marker word.</t>
+          <t>The label segments that mark an interface or VLAN address.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B21" s="2" t="inlineStr"/>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">            if (segment == w)
-                return true;</t>
+          <t xml:space="preserve">    var evidence = false;</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>The segment is the word itself ("vlan").</t>
+          <t>Set to true as soon as one piece of evidence is found.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B22" s="2" t="inlineStr"/>
       <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            if (segment.indexOf(w) == 0 &amp;&amp; /^[0-9]+$/.test(segment.substring(w.length)))
-                return true;</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>The segment is the word followed by digits only ("vlan705", "v201").</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="2" t="inlineStr"/>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            if (w.length &gt;= 3 &amp;&amp; segment.length &gt; w.length &amp;&amp; segment.substring(segment.length - w.length) == w)
-                return true;</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>For words of three letters or more, the segment ends in the word ("multihostvip").</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="2" t="inlineStr"/>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        }</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>End of the block.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="2" t="inlineStr"/>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        return false;</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>No marker word fits this segment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="2" t="inlineStr"/>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    }</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>End of the block.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr"/>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Interface evidence first</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr"/>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>The rule goes on only when the DNS domain contains a listed interface domain or one of the segments after the first is a listed marker. Plenty of ordinary server names contain hyphens ("ah-1047132-001"); without this check the prefix walk would strip real hostnames and could land on an unrelated device.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="B28" s="2" t="inlineStr"/>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    var domains = list('usem.ci_lookup.interface_domains', '.network.');</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Interface domains, from the property.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="B29" s="2" t="inlineStr"/>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    var markers = list('usem.ci_lookup.interface_markers', 'vlan,v,hsrp,vrrp,po,eth,gi,te,lo,mgmt,aom,vs,fab');</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>Interface marker words, from the property.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="B30" s="2" t="inlineStr"/>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    var evidence = false;</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>Set to true as soon as one piece of evidence is found.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="B31" s="2" t="inlineStr"/>
-      <c r="C31" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">    for (var d = 0; d &lt; domains.length; d++)
         if (full.indexOf(domains[d]) != -1)
             evidence = true;</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Evidence when the DNS name contains a listed interface domain.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="B32" s="2" t="inlineStr"/>
-      <c r="C32" s="3" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">    for (var s = 1; s &lt; segments.length; s++)
         if (isMarker(segments[s], markers))
             evidence = true;</t>
         </is>
       </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Evidence when a segment after the first is a listed marker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (!evidence)
+        return null;</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>No evidence -&gt; this host is not one the rule is for; decline untouched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr"/>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Walk the prefixes from the longest to the shortest</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr"/>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>One segment is dropped from the right at a time and the prefix is searched as a device name. The device name is the leading part of the label but its length varies by site, and trying the longest prefix first keeps "site-device-01" from being cut down to "site" when a CI with the longer name exists. The first prefix that finds anything decides: one CI is the match, two CIs mean the rule declines. Network devices live in two branches of the CMDB, Network Gear (switches, routers, firewalls) and Load Balancer, which the platform files under Server; both are searched and the hits are counted together.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    var tables = ['cmdb_ci_netgear', 'cmdb_ci_lb'];</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>The two branches that hold network devices.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    for (var k = segments.length - 1; k &gt;= 1; k--) {</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>From the longest prefix (all segments but the last) down to the first segment alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        var base = segments.slice(0, k).join('-');</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>longest prefix first, e.g. "uspaltwrr01drm0119-cz04-hsrp"</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        var hits = [];</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Devices named exactly like this prefix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        for (var t = 0; t &lt; tables.length; t++) {</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Search both branches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            var gr = new GlideRecord(tables[t]);</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Search on one branch and every class beneath it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            if (!gr.isValid())
+                continue;</t>
+        </is>
+      </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Evidence when a segment after the first is a listed marker.</t>
+          <t>The class is not installed on this instance -&gt; decline rather than fail.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B33" s="2" t="inlineStr"/>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    if (!evidence)
-        return null;</t>
+          <t xml:space="preserve">            gr.addQuery('name', base);</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>No evidence -&gt; this host is not one the rule is for; decline untouched.</t>
+          <t>Condition: name equals the derived name.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr"/>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>Walk the prefixes from the longest to the shortest</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr"/>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>One segment is dropped from the right at a time and the prefix is searched as a device name. The device name is the leading part of the label but its length varies by site, and trying the longest prefix first keeps "site-device-01" from being cut down to "site" when a CI with the longer name exists. The first prefix that finds anything decides: one CI is the match, two CIs mean the rule declines. Network devices live in two branches of the CMDB, Network Gear (switches, routers, firewalls) and Load Balancer, which the platform files under Server; both are searched and the hits are counted together.</t>
+      <c r="A34" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr"/>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            if (ignore)
+                gr.addQuery('sys_class_name', 'NOT IN', ignore);</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>When the ignore list is filled, exclude those classes from the search.</t>
         </is>
       </c>
     </row>
@@ -3996,12 +3852,12 @@
       <c r="B35" s="2" t="inlineStr"/>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    var tables = ['cmdb_ci_netgear', 'cmdb_ci_lb'];</t>
+          <t xml:space="preserve">            gr.query();</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>The two branches that hold network devices.</t>
+          <t>Runs the search.</t>
         </is>
       </c>
     </row>
@@ -4012,12 +3868,13 @@
       <c r="B36" s="2" t="inlineStr"/>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    for (var k = segments.length - 1; k &gt;= 1; k--) {</t>
+          <t xml:space="preserve">            while (gr.next() &amp;&amp; hits.length &lt; 2)
+                hits.push(gr.getUniqueValue());</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>From the longest prefix (all segments but the last) down to the first segment alone.</t>
+          <t>Collect up to two hits; two is already one too many.</t>
         </is>
       </c>
     </row>
@@ -4028,12 +3885,12 @@
       <c r="B37" s="2" t="inlineStr"/>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        var base = segments.slice(0, k).join('-');</t>
+          <t xml:space="preserve">        }</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>longest prefix first, e.g. "uspaltwrr01drm0119-cz04-hsrp"</t>
+          <t>End of the block.</t>
         </is>
       </c>
     </row>
@@ -4044,12 +3901,13 @@
       <c r="B38" s="2" t="inlineStr"/>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        var hits = [];</t>
+          <t xml:space="preserve">        if (hits.length == 0)
+            continue;</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Devices named exactly like this prefix.</t>
+          <t>nothing named like this, try a shorter prefix</t>
         </is>
       </c>
     </row>
@@ -4060,12 +3918,13 @@
       <c r="B39" s="2" t="inlineStr"/>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        for (var t = 0; t &lt; tables.length; t++) {</t>
+          <t xml:space="preserve">        if (hits.length &gt; 1)
+            return null;</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Search both branches.</t>
+          <t>two devices carry this name, never guess</t>
         </is>
       </c>
     </row>
@@ -4076,12 +3935,12 @@
       <c r="B40" s="2" t="inlineStr"/>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">            var gr = new GlideRecord(tables[t]);</t>
+          <t xml:space="preserve">        return hits[0];</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Search on one branch and every class beneath it.</t>
+          <t>Exactly one device carries this prefix -&gt; match.</t>
         </is>
       </c>
     </row>
@@ -4092,13 +3951,12 @@
       <c r="B41" s="2" t="inlineStr"/>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">            if (!gr.isValid())
-                continue;</t>
+          <t xml:space="preserve">    }</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>The class is not installed on this instance -&gt; decline rather than fail.</t>
+          <t>End of the block.</t>
         </is>
       </c>
     </row>
@@ -4109,12 +3967,12 @@
       <c r="B42" s="2" t="inlineStr"/>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">            gr.addQuery('name', base);</t>
+          <t xml:space="preserve">    return null;</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Condition: name equals the derived name.</t>
+          <t>Nothing usable -&gt; decline; the next rule gets its turn.</t>
         </is>
       </c>
     </row>
@@ -4125,158 +3983,10 @@
       <c r="B43" s="2" t="inlineStr"/>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">            if (ignore)
-                gr.addQuery('sys_class_name', 'NOT IN', ignore);</t>
+          <t>})(rule, sourceValue, sourcePayload);</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>When the ignore list is filled, exclude those classes from the search.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="n">
-        <v>41</v>
-      </c>
-      <c r="B44" s="2" t="inlineStr"/>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            gr.query();</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>Runs the search.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="n">
-        <v>42</v>
-      </c>
-      <c r="B45" s="2" t="inlineStr"/>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            while (gr.next() &amp;&amp; hits.length &lt; 2)
-                hits.push(gr.getUniqueValue());</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>Collect up to two hits; two is already one too many.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="n">
-        <v>43</v>
-      </c>
-      <c r="B46" s="2" t="inlineStr"/>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        }</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>End of the block.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="B47" s="2" t="inlineStr"/>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        if (hits.length == 0)
-            continue;</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>nothing named like this, try a shorter prefix</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="B48" s="2" t="inlineStr"/>
-      <c r="C48" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        if (hits.length &gt; 1)
-            return null;</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>two devices carry this name, never guess</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="n">
-        <v>46</v>
-      </c>
-      <c r="B49" s="2" t="inlineStr"/>
-      <c r="C49" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        return hits[0];</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>Exactly one device carries this prefix -&gt; match.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="n">
-        <v>47</v>
-      </c>
-      <c r="B50" s="2" t="inlineStr"/>
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    }</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>End of the block.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="B51" s="2" t="inlineStr"/>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    return null;</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>Nothing usable -&gt; decline; the next rule gets its turn.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="B52" s="2" t="inlineStr"/>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>})(rule, sourceValue, sourcePayload);</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>Runs the function immediately with the values the framework supplied.</t>
         </is>
@@ -4579,7 +4289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D56"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4748,12 +4458,12 @@
       <c r="B10" s="2" t="inlineStr"/>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    function list(name, fallback) {</t>
+          <t xml:space="preserve">    function isMarker(segment, words) {</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>list() reads a comma separated system property into a lower-cased list, falling back to the default shipped with the rule; the lists are tuned in the properties, not in the script.</t>
+          <t>isMarker() says whether one hyphen segment of the label is a listed marker: the word itself ("vlan"), the word followed by digits only ("vlan705", "v201"), or, for words of three letters or more, a segment ending in the word ("multihostvip").</t>
         </is>
       </c>
     </row>
@@ -4764,12 +4474,12 @@
       <c r="B11" s="2" t="inlineStr"/>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        var parts = ('' + gs.getProperty(name, fallback)).split(',');</t>
+          <t xml:space="preserve">        for (var i = 0; i &lt; words.length; i++) {</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Read the property (or the default shipped with the rule) and split it on commas.</t>
+          <t>Loop over the listed marker words.</t>
         </is>
       </c>
     </row>
@@ -4780,12 +4490,12 @@
       <c r="B12" s="2" t="inlineStr"/>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        var out = [];</t>
+          <t xml:space="preserve">            var w = words[i];</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>The cleaned list.</t>
+          <t>One marker word.</t>
         </is>
       </c>
     </row>
@@ -4796,12 +4506,13 @@
       <c r="B13" s="2" t="inlineStr"/>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        for (var i = 0; i &lt; parts.length; i++) {</t>
+          <t xml:space="preserve">            if (segment == w)
+                return true;</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Loop over the comma separated entries.</t>
+          <t>The segment is the word itself ("vlan").</t>
         </is>
       </c>
     </row>
@@ -4812,12 +4523,13 @@
       <c r="B14" s="2" t="inlineStr"/>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">            var item = parts[i].trim().toLowerCase();</t>
+          <t xml:space="preserve">            if (segment.indexOf(w) == 0 &amp;&amp; /^[0-9]+$/.test(segment.substring(w.length)))
+                return true;</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Trim and lower-case one entry.</t>
+          <t>The segment is the word followed by digits only ("vlan705", "v201").</t>
         </is>
       </c>
     </row>
@@ -4828,13 +4540,13 @@
       <c r="B15" s="2" t="inlineStr"/>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">            if (item)
-                out.push(item);</t>
+          <t xml:space="preserve">            if (w.length &gt;= 3 &amp;&amp; segment.length &gt; w.length &amp;&amp; segment.substring(segment.length - w.length) == w)
+                return true;</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Keep non-empty entries.</t>
+          <t>For words of three letters or more, the segment ends in the word ("multihostvip").</t>
         </is>
       </c>
     </row>
@@ -4861,12 +4573,12 @@
       <c r="B17" s="2" t="inlineStr"/>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        return out;</t>
+          <t xml:space="preserve">        return false;</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>The list of lower-cased entries.</t>
+          <t>No marker word fits this segment.</t>
         </is>
       </c>
     </row>
@@ -4887,294 +4599,295 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="2" t="inlineStr"/>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    function isMarker(segment, words) {</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>isMarker() says whether one hyphen segment of the label is a listed marker: the word itself ("vlan"), the word followed by digits only ("vlan705", "v201"), or, for words of three letters or more, a segment ending in the word ("multihostvip").</t>
+      <c r="A19" s="4" t="inlineStr"/>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>VIP evidence first</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr"/>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>The rule goes on only when the OS text contains a listed load balancer word or one of the label segments is a listed VIP marker. A Load Balancer Service must never be returned for an ordinary server that happens to share an address with a VIP; this check keeps the rule to the hosts that really are VIPs ("f5 big ip", "rbps-dev3-sve-vip"). The load balancer products looked for in the OS text, and the label segments that mark a virtual IP. Extend these two lists when a site uses another naming habit.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" s="2" t="inlineStr"/>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        for (var i = 0; i &lt; words.length; i++) {</t>
+          <t xml:space="preserve">    var osMarkers = ['f5', 'big-ip', 'big ip', 'netscaler'];</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Loop over the listed marker words.</t>
+          <t>The load balancer products looked for in the OS text.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B21" s="2" t="inlineStr"/>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">            var w = words[i];</t>
+          <t xml:space="preserve">    var labelMarkers = ['vip', 'vs'];</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>One marker word.</t>
+          <t>The label segments that mark a virtual IP.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B22" s="2" t="inlineStr"/>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">            if (segment == w)
-                return true;</t>
+          <t xml:space="preserve">    var evidence = false;</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>The segment is the word itself ("vlan").</t>
+          <t>Set to true as soon as one piece of evidence is found.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B23" s="2" t="inlineStr"/>
       <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            if (segment.indexOf(w) == 0 &amp;&amp; /^[0-9]+$/.test(segment.substring(w.length)))
-                return true;</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>The segment is the word followed by digits only ("vlan705", "v201").</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="2" t="inlineStr"/>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            if (w.length &gt;= 3 &amp;&amp; segment.length &gt; w.length &amp;&amp; segment.substring(segment.length - w.length) == w)
-                return true;</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>For words of three letters or more, the segment ends in the word ("multihostvip").</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="2" t="inlineStr"/>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        }</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>End of the block.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="2" t="inlineStr"/>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        return false;</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>No marker word fits this segment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="2" t="inlineStr"/>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    }</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>End of the block.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr"/>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>VIP evidence first</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr"/>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>The rule goes on only when the OS text contains a listed load balancer word or one of the label segments is a listed VIP marker. A Load Balancer Service must never be returned for an ordinary server that happens to share an address with a VIP; this check keeps the rule to the hosts that really are VIPs ("f5 big ip", "rbps-dev3-sve-vip").</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="B29" s="2" t="inlineStr"/>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    var osMarkers = list('usem.ci_lookup.vip_os_markers', 'f5,big-ip,big ip,netscaler');</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>Load balancer product words looked for in the OS text, from the property.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="B30" s="2" t="inlineStr"/>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    var labelMarkers = list('usem.ci_lookup.vip_markers', 'vip,vs');</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>VIP marker words for the label segments, from the property.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="B31" s="2" t="inlineStr"/>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    var evidence = false;</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>Set to true as soon as one piece of evidence is found.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="B32" s="2" t="inlineStr"/>
-      <c r="C32" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">    for (var m = 0; m &lt; osMarkers.length; m++)
         if (os.indexOf(osMarkers[m]) != -1)
             evidence = true;</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Evidence when the OS text contains a listed load balancer word.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="B33" s="2" t="inlineStr"/>
-      <c r="C33" s="3" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">    var segments = label ? label.split('-') : [];</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>The hyphen segments of the label; none without a DNS name.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="B34" s="2" t="inlineStr"/>
-      <c r="C34" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">    for (var s = 0; s &lt; segments.length; s++)
         if (isMarker(segments[s], labelMarkers))
             evidence = true;</t>
         </is>
       </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Evidence when any segment is a listed VIP marker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    if (!evidence)
+        return null;</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>No evidence -&gt; this host is not one the rule is for; decline untouched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr"/>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>The one service, by fqdn, then name, then address</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr"/>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>The scanned DNS name is tried in the fqdn field, then in the name field, then the label in the name field, then the scanned address in ip_address. Each step accepts exactly one service; a step that finds two ends the rule with null, because a weaker piece of evidence could otherwise pick a different service; a step that finds nothing hands over to the next.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    function one(field, value) {</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Helper: the one Load Balancer Service whose field equals the value; undefined when nothing to search or nothing found, null when two are found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        if (!value)
+            return undefined;</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>nothing to search, next step</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        var gr = new GlideRecord('cmdb_ci_lb_service');</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Search on the Load Balancer Service class and every class beneath it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        if (!gr.isValid())
+            return null;</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>class not installed here, decline</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        gr.addQuery(field, value);</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Condition: the field named by the step equals the value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        if (ignore)
+            gr.addQuery('sys_class_name', 'NOT IN', ignore);</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>When the ignore list is filled, exclude those classes from the search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr"/>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        gr.query();</t>
+        </is>
+      </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Evidence when any segment is a listed VIP marker.</t>
+          <t>Runs the search.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B35" s="2" t="inlineStr"/>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    if (!evidence)
-        return null;</t>
+          <t xml:space="preserve">        if (!gr.next())
+            return undefined;</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>No evidence -&gt; this host is not one the rule is for; decline untouched.</t>
+          <t>nothing found, next step</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr"/>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>The one service, by fqdn, then name, then address</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr"/>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>The scanned DNS name is tried in the fqdn field, then in the name field, then the label in the name field, then the scanned address in ip_address. Each step accepts exactly one service; a step that finds two ends the rule with null, because a weaker piece of evidence could otherwise pick a different service; a step that finds nothing hands over to the next.</t>
+      <c r="A36" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr"/>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        var id = gr.getUniqueValue();</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>The sys_id of the CI found.</t>
         </is>
       </c>
     </row>
@@ -5185,12 +4898,13 @@
       <c r="B37" s="2" t="inlineStr"/>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    function one(field, value) {</t>
+          <t xml:space="preserve">        if (gr.hasNext())
+            return null;</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Helper: the one Load Balancer Service whose field equals the value; undefined when nothing to search or nothing found, null when two are found.</t>
+          <t>two services, never guess</t>
         </is>
       </c>
     </row>
@@ -5201,13 +4915,12 @@
       <c r="B38" s="2" t="inlineStr"/>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        if (!value)
-            return undefined;</t>
+          <t xml:space="preserve">        return id;</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>nothing to search, next step</t>
+          <t>The CI passed every check -&gt; its sys_id goes back to the framework.</t>
         </is>
       </c>
     </row>
@@ -5218,12 +4931,12 @@
       <c r="B39" s="2" t="inlineStr"/>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        var gr = new GlideRecord('cmdb_ci_lb_service');</t>
+          <t xml:space="preserve">    }</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Search on the Load Balancer Service class and every class beneath it.</t>
+          <t>End of the block.</t>
         </is>
       </c>
     </row>
@@ -5234,13 +4947,12 @@
       <c r="B40" s="2" t="inlineStr"/>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        if (!gr.isValid())
-            return null;</t>
+          <t xml:space="preserve">    var steps = [['fqdn', dns], ['name', dns], ['name', label], ['ip_address', ip]];</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>class not installed here, decline</t>
+          <t>The evidence in order of strength: the DNS name as fqdn, as name, its label as name, then the address.</t>
         </is>
       </c>
     </row>
@@ -5251,12 +4963,12 @@
       <c r="B41" s="2" t="inlineStr"/>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        gr.addQuery(field, value);</t>
+          <t xml:space="preserve">    for (var t = 0; t &lt; steps.length; t++) {</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Condition: the field named by the step equals the value.</t>
+          <t>Try the steps in order.</t>
         </is>
       </c>
     </row>
@@ -5267,13 +4979,12 @@
       <c r="B42" s="2" t="inlineStr"/>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        if (ignore)
-            gr.addQuery('sys_class_name', 'NOT IN', ignore);</t>
+          <t xml:space="preserve">        var found = one(steps[t][0], steps[t][1]);</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>When the ignore list is filled, exclude those classes from the search.</t>
+          <t>Run one step.</t>
         </is>
       </c>
     </row>
@@ -5284,12 +4995,13 @@
       <c r="B43" s="2" t="inlineStr"/>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        gr.query();</t>
+          <t xml:space="preserve">        if (found === null)
+            return null;</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Runs the search.</t>
+          <t>Two services at this step -&gt; decline; a weaker step must not override an ambiguous stronger one.</t>
         </is>
       </c>
     </row>
@@ -5300,13 +5012,13 @@
       <c r="B44" s="2" t="inlineStr"/>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        if (!gr.next())
-            return undefined;</t>
+          <t xml:space="preserve">        if (found)
+            return found;</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>nothing found, next step</t>
+          <t>Exactly one service -&gt; match.</t>
         </is>
       </c>
     </row>
@@ -5317,12 +5029,12 @@
       <c r="B45" s="2" t="inlineStr"/>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        var id = gr.getUniqueValue();</t>
+          <t xml:space="preserve">    }</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>The sys_id of the CI found.</t>
+          <t>End of the block.</t>
         </is>
       </c>
     </row>
@@ -5333,13 +5045,12 @@
       <c r="B46" s="2" t="inlineStr"/>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        if (gr.hasNext())
-            return null;</t>
+          <t xml:space="preserve">    return null;</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>two services, never guess</t>
+          <t>Nothing usable -&gt; decline; the next rule gets its turn.</t>
         </is>
       </c>
     </row>
@@ -5350,156 +5061,10 @@
       <c r="B47" s="2" t="inlineStr"/>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">        return id;</t>
+          <t>})(rule, sourceValue, sourcePayload);</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>The CI passed every check -&gt; its sys_id goes back to the framework.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="B48" s="2" t="inlineStr"/>
-      <c r="C48" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    }</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>End of the block.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="n">
-        <v>46</v>
-      </c>
-      <c r="B49" s="2" t="inlineStr"/>
-      <c r="C49" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    var steps = [['fqdn', dns], ['name', dns], ['name', label], ['ip_address', ip]];</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>The evidence in order of strength: the DNS name as fqdn, as name, its label as name, then the address.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="n">
-        <v>47</v>
-      </c>
-      <c r="B50" s="2" t="inlineStr"/>
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    for (var t = 0; t &lt; steps.length; t++) {</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>Try the steps in order.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="B51" s="2" t="inlineStr"/>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        var found = one(steps[t][0], steps[t][1]);</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>Run one step.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="B52" s="2" t="inlineStr"/>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        if (found === null)
-            return null;</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>Two services at this step -&gt; decline; a weaker step must not override an ambiguous stronger one.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="B53" s="2" t="inlineStr"/>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        if (found)
-            return found;</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>Exactly one service -&gt; match.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="B54" s="2" t="inlineStr"/>
-      <c r="C54" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    }</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>End of the block.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="n">
-        <v>52</v>
-      </c>
-      <c r="B55" s="2" t="inlineStr"/>
-      <c r="C55" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    return null;</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>Nothing usable -&gt; decline; the next rule gets its turn.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="B56" s="2" t="inlineStr"/>
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t>})(rule, sourceValue, sourcePayload);</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>Runs the function immediately with the values the framework supplied.</t>
         </is>

</xml_diff>

<commit_message>
Qualys CI lookup rules V2.4 / V3.4: sample payload back in every header, each stage note walks the sample through; comments only
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UaiSzs85tKmfaeLA1rAxsP
</commit_message>
<xml_diff>
--- a/stories/qualys-ci-lookup-rules/Qualys CI Lookup Rules - Code Line Explanations.xlsx
+++ b/stories/qualys-ci-lookup-rules/Qualys CI Lookup Rules - Code Line Explanations.xlsx
@@ -29,7 +29,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="850 FQDN Name Broad Match" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overview'!$A$1:$I$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overview'!$A$1:$K$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -492,18 +492,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -529,25 +531,35 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Sample payload</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Returns</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Expected for the sample</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Runs before it</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Which hosts reach it</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Runs after it</t>
         </is>
@@ -572,27 +584,44 @@
           <t>Serial number first. A serial stays with a machine for its whole life while names and addresses get reused, so it is the strongest identifier Qualys gives us. This rule trusts it only inside the CMDB class the scanned OS points at.</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>sourceValue is the SERIAL_NUMBER field; the rule also reads the OS from sourcePayload.</t>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "35832680",
+  "IP": "171.128.225.96",
+  "TRACKING_METHOD": "AGENT",
+  "OS": "Red Hat Enterprise Linux 9.8",
+  "DNS": "ah-1047132-001.sdi.corp.bankofamerica.com",
+  "SERIAL_NUMBER": "VMware-42 1a 9c 3f 7d 2e 61 b8-55 04 e2 91 6a 27 c3 08"
+}</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>sourceValue is the SERIAL_NUMBER field, "VMware-42 1a 9c 3f 7d 2e 61 b8-55 04 e2 91 6a 27 c3 08"; the rule also reads the OS from sourcePayload.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
           <t>the sys_id of the one CI of that class whose serial_number equals the scanned serial; null when none or more than one carries it.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>the Linux Server CI "ah-1047132-001", whose serial_number holds the same serial; null when no Linux Server carries it, or two do.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>nothing custom runs before this rule.</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>every host that reports a serial. In our feed that is the Cloud Agent hosts; the unauthenticated network scans rarely carry one.</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>USEM Serial Number Hardware Match repeats the search across the whole hardware tree for hosts whose OS gives no class or whose CI is classed differently.</t>
         </is>
@@ -617,27 +646,44 @@
           <t>Second and last serial rule: the same serial search, but across the whole hardware tree (servers, computers, network gear, storage, printers). It exists for hosts whose OS gives no usable class and for CIs that sit in a different class than the OS suggests.</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>sourceValue is the SERIAL_NUMBER field.</t>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "35920204",
+  "IP": "171.135.28.125",
+  "TRACKING_METHOD": "IP",
+  "OS": "Ubuntu / Tiny Core Linux / Linux 2.6.x / IBM ASM / HP StoreOnce / F5 Networks Big-IP / Cisco IOS Software",
+  "DNS": "txr9gxcenah031.sdi.corp.bankofamerica.com",
+  "SERIAL_NUMBER": "MXQ13005TC"
+}</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>sourceValue is the SERIAL_NUMBER field, "MXQ13005TC".</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
           <t>the sys_id of the one hardware CI whose serial_number equals the scanned serial; null when none or more than one carries it.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>USEM Serial Number Class Match already tried the serial inside the class the OS implies.</t>
-        </is>
-      </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>hosts with a serial whose OS is unknown (an unauthenticated scan listing several guesses, such as "Ubuntu / Tiny Core Linux / Linux 2.6.x / IBM ASM / HP StoreOnce / F5 Networks Big-IP / Cisco IOS Software") or whose CI is classed differently.</t>
+          <t>the Server CI "txr9gxcenah031", kept in the generic Server class because the scan could not identify its OS; its serial_number is "MXQ13005TC".</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>USEM Serial Number Class Match already tried the serial inside the class the OS implies; the sample OS is a list of seven guesses, so that rule declined without searching.</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>hosts with a serial whose OS is unknown (an unauthenticated scan listing several guesses, as in the sample) or whose CI is classed differently.</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>the phone rule and the name rules. A serial that is not unique in the whole hardware tree is never used.</t>
         </is>
@@ -662,27 +708,43 @@
           <t>Cisco Unified Communications Manager names every phone "SEP" followed by its MAC address, and Qualys reports that name as the DNS label (under voip.bankofamerica.com in our feed). The rule turns the label back into a MAC address and looks for exactly one IP Phone CI that carries it.</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>sourceValue is the DNS field.</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "41277345",
+  "IP": "30.144.62.108",
+  "TRACKING_METHOD": "IP",
+  "OS": "Cisco IP Phone",
+  "DNS": "sep64f69dd5c9b0.voip.bankofamerica.com"
+}</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
+          <t>sourceValue is the DNS field, "sep64f69dd5c9b0.voip.bankofamerica.com".</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
           <t>the sys_id of the IP Phone CI whose network adapter, mac_address field or name carries that MAC; null for any label that is not a phone label, and when no phone or two phones carry the MAC.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>the IP Phone CI "SEP64F69DD5C9B0", found through the adapter that carries the MAC 64:F6:9D:D5:C9:B0.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>the serial number rules (phones report none).</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>only hosts whose DNS label is "sep" plus twelve hexadecimal characters; every other host passes through untouched.</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>the FQDN and hostname rules. Phones are resolved before them so a phone label is never tried as a server name, and because only IP Phone CIs are searched a MAC clash can never pull in a switch or a server.</t>
         </is>
@@ -707,27 +769,43 @@
           <t>The first name rule: the scanned DNS name against the fqdn field of a CI, inside the class the scanned OS points at. An exact FQDN on the CI is the most precise name evidence we have, so it comes before any hostname matching.</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>sourceValue is the DNS field; the rule also reads the OS and the IP from sourcePayload.</t>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "83047612",
+  "IP": "30.206.199.36",
+  "TRACKING_METHOD": "IP",
+  "OS": "VMware ESXi 7.0.3 build 24723872",
+  "DNS": "vsdnac22xsdi004.sdi.corp.bankofamerica.com"
+}</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
+          <t>sourceValue is the DNS field, "vsdnac22xsdi004.sdi.corp.bankofamerica.com"; the rule also reads the OS and the IP from sourcePayload.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
           <t>the sys_id of the one CI of that class whose fqdn equals the scanned name; with duplicate fqdn values, the one that also carries the scanned IP; null otherwise.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>the ESX Server CI "vsdnac22xsdi004", whose fqdn is the scanned name; two ESX Servers with that fqdn are accepted only when exactly one also carries the IP 30.206.199.36.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>the serial number rules and the IP phone rule found nothing.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>every host with a dotted DNS name, which is the bulk of the Qualys feed.</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>USEM FQDN Hardware Match repeats the exact FQDN search across every hardware class; the hostname-plus-domain rules and then the plain hostname rules follow.</t>
         </is>
@@ -752,27 +830,43 @@
           <t>The exact FQDN search again, across the whole hardware tree. It picks up the hosts whose OS gives no class and the CIs kept in a generic or different class than the OS suggests.</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>sourceValue is the DNS field; the rule also reads the IP from sourcePayload.</t>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "35920204",
+  "IP": "171.135.28.125",
+  "TRACKING_METHOD": "IP",
+  "OS": "Ubuntu / Tiny Core Linux / Linux 2.6.x / IBM ASM / HP StoreOnce / F5 Networks Big-IP / Cisco IOS Software",
+  "DNS": "txr9gxcenah031.sdi.corp.bankofamerica.com"
+}</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
+          <t>sourceValue is the DNS field, "txr9gxcenah031.sdi.corp.bankofamerica.com"; the rule also reads the IP from sourcePayload.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
           <t>the sys_id of the one hardware CI whose fqdn equals the scanned name; with duplicates, the one that also carries the scanned IP; null otherwise.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>USEM FQDN Class Match tried the exact FQDN inside the class the OS implies.</t>
-        </is>
-      </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>hosts whose OS gives no class (unauthenticated scans with a multi-guess OS) or whose CI is classed differently from the OS.</t>
+          <t>the Server CI "txr9gxcenah031" whose fqdn is the scanned name; duplicates are resolved by the IP 171.135.28.125 or declined.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>USEM FQDN Class Match tried the exact FQDN inside the class the OS implies; the sample OS is a list of seven guesses, so that rule declined without searching.</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>hosts whose OS gives no class (unauthenticated scans with a multi-guess OS, as in the sample) or whose CI is classed differently from the OS.</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>the hostname-plus-domain rules, for CIs that carry no fqdn value at all.</t>
         </is>
@@ -797,27 +891,44 @@
           <t>For CIs that are named with the short hostname and carry the domain in another field (dns_domain, or an fqdn that was never copied into the name). The short name and the domain are matched together, inside the class the scanned OS points at.</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>sourceValue is the DNS field; the rule also reads the OS and the IP from sourcePayload.</t>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "35832680",
+  "IP": "171.128.225.96",
+  "TRACKING_METHOD": "AGENT",
+  "OS": "Red Hat Enterprise Linux 9.8",
+  "DNS": "ah-1047132-001.sdi.corp.bankofamerica.com",
+  "QG_HOSTID": "633769a4-0139-0002-e352-005056bf41ea"
+}</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
+          <t>sourceValue is the DNS field, "ah-1047132-001.sdi.corp.bankofamerica.com"; the rule also reads the OS and the IP from sourcePayload.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
           <t>the sys_id of the one CI of that class named with the short hostname whose own domain information agrees with the scanned domain; a namesake in another domain is never picked.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>the Linux Server CI named "ah-1047132-001" whose dns_domain is "sdi.corp.bankofamerica.com".</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>the FQDN rules looked for the exact name in the fqdn field and found nothing.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>hosts whose CI has no exact fqdn value but is named with the short hostname and shows the domain elsewhere.</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>USEM Hostname Domain Hardware Match repeats the search across all hardware, USEM Layered DNS Match reads the discovery DNS records, and the plain hostname rules accept a unique short name without domain evidence.</t>
         </is>
@@ -842,27 +953,43 @@
           <t>Short hostname plus domain evidence again, across the whole hardware tree, for CIs classed generically (Server, Computer) or differently from the scanned OS.</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>sourceValue is the DNS field; the rule also reads the IP from sourcePayload.</t>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "35884392",
+  "IP": "171.128.140.192",
+  "TRACKING_METHOD": "IP",
+  "OS": "Ubuntu/Linux",
+  "DNS": "lrche01xtrapd01.sdi.corp.bankofamerica.com"
+}</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
+          <t>sourceValue is the DNS field, "lrche01xtrapd01.sdi.corp.bankofamerica.com"; the rule also reads the IP from sourcePayload.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
           <t>the sys_id of the one hardware CI named with the short hostname whose fqdn or dns_domain agrees with the scanned domain; null otherwise.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>USEM Hostname Domain Class Match tried the same evidence inside the class the OS implies.</t>
-        </is>
-      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
+          <t>the CI named "lrche01xtrapd01" in the generic Server class, whose fqdn is the scanned name.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>USEM Hostname Domain Class Match tried the same evidence inside the class the OS implies (Linux Server for "Ubuntu/Linux") and found nothing, because the CI sits in the generic Server class.</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
           <t>hosts whose CI is classed generically or differently from the scanned OS, so the class-scoped search found nothing.</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>USEM Layered DNS Match and then the plain hostname rules.</t>
         </is>
@@ -887,27 +1014,44 @@
           <t>Discovery keeps names and addresses as their own records linked to the device: a DNS Name record is tied to an IP Address record, the IP Address record belongs to a Network Adapter, and the adapter belongs to the CI. This rule follows that chain, which is the only way to find a host whose name is not written on the CI record at all, and it resolves aliases to the real machine.</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>sourceValue is the DNS field; the rule also reads the IP from sourcePayload.</t>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "42773078",
+  "IP": "167.202.60.26",
+  "TRACKING_METHOD": "IP",
+  "OS": "Red Hat Enterprise Linux Server 7.9",
+  "DNS": "hklvteqoradbp3.hk.baml.com",
+  "QG_HOSTID": "6337dede-02e7-0002-ad2c-0050569765df"
+}</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
+          <t>sourceValue is the DNS field, "hklvteqoradbp3.hk.baml.com"; the rule also reads the IP from sourcePayload.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
           <t>the sys_id of the CI at the end of the chain DNS Name -&gt; IP Address -&gt; adapter -&gt; CI; when several CIs answer to the name, the one whose chain runs through the scanned IP; null otherwise.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>the Linux Server "hklvteqoradbp3", reached through DNS Name "hklvteqoradbp3.hk.baml.com" -&gt; IP Address "167.202.60.26" -&gt; adapter "eth0".</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>the FQDN and hostname-plus-domain rules looked at name fields stored on the CI record itself.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>hosts whose name lives only in the discovery DNS records, and aliases that point at an address of the device.</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>the plain hostname rules and USEM FQDN Name Hardware Match.</t>
         </is>
@@ -932,27 +1076,44 @@
           <t>The short hostname alone, inside the class the scanned OS points at. For CIs that carry only a short name and no domain information; the agreement between CI class and scanned OS stands in for the missing domain evidence.</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>sourceValue is the DNS field; the rule also reads the OS from sourcePayload.</t>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "35850078",
+  "IP": "30.143.70.11",
+  "TRACKING_METHOD": "IP",
+  "OS": "Windows Server 2016 Standard 64 bit Edition Version 1607",
+  "DNS": "wsaoi01zeapd1.sdi.corp.bankofamerica.com",
+  "NETBIOS": "WSAOI01ZEAPD1"
+}</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
+          <t>sourceValue is the DNS field, "wsaoi01zeapd1.sdi.corp.bankofamerica.com"; the rule also reads the OS from sourcePayload.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
           <t>the sys_id of the one CI of that class named with the short hostname (names compare case-insensitively); null when none or two carry it.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>the Windows Server CI named "WSAOI01ZEAPD1"; a second Windows Server with the same name would make the rule decline.</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>every rule so far needed domain evidence on the CI (fqdn, dns_domain or the discovery DNS records).</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>hosts whose CI carries only a short name and no domain information at all.</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>USEM Hostname Hardware Match repeats the short name search across all hardware with a class sanity check; USEM FQDN Name Hardware Match handles CIs named with the full FQDN.</t>
         </is>
@@ -977,27 +1138,44 @@
           <t>The short hostname across the whole hardware tree, with a check that the CI found does not contradict the scanned OS. For CIs classed generically (Server, Computer, UNIX Server) or differently from the OS.</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>sourceValue is the DNS field; the rule also reads the OS from sourcePayload.</t>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "80217765",
+  "IP": "171.150.219.123",
+  "TRACKING_METHOD": "IP",
+  "OS": "AIX 7.3 TL3",
+  "DNS": "va2ausapabw0.bankofamerica.com",
+  "QG_HOSTID": "6337e0dc-007d-0002-c47d-005056a4fcd5"
+}</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
+          <t>sourceValue is the DNS field, "va2ausapabw0.bankofamerica.com"; the rule also reads the OS from sourcePayload.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
           <t>the sys_id of the one hardware CI named with the short hostname, accepted when its class agrees with the scanned OS or is generic; null when the name is shared or the class contradicts the scan.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>USEM Hostname Class Match required the short name to be unique inside the class the OS implies.</t>
-        </is>
-      </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
+          <t>the CI named "va2ausapabw0" in the generic Server class; it would also be accepted as an AIX Server, and rejected as, say, a Windows Server.</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>USEM Hostname Class Match required the short name to be unique inside the class the OS implies (AIX Server) and found nothing there.</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
           <t>hosts whose CI is classed generically or whose OS gave no class.</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>USEM FQDN Name Hardware Match, then the IP address rules for hosts without a usable name.</t>
         </is>
@@ -1022,27 +1200,43 @@
           <t>Server management controllers (HP iLO, Oracle ILOM, Dell iDRAC, IBM IMM, Cisco CIMC, generic BMC or IPMI) are scanned under their own DNS label, which is the server name plus a suffix such as "-ilo", "-ilom" or "-idrac", so the name rules never find them. The findings belong to the server, and this rule strips the suffix and matches the server.</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>sourceValue is the DNS field; the rule also reads the OS from sourcePayload.</t>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "1201534877",
+  "IP": "159.185.200.11",
+  "TRACKING_METHOD": "IP",
+  "OS": "HP iLO",
+  "DNS": "tx6dd630001-ilo.bankofamerica.com"
+}</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
+          <t>sourceValue is the DNS field, "tx6dd630001-ilo.bankofamerica.com"; the rule also reads the OS from sourcePayload.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
           <t>the sys_id of the one hardware CI named like the label without its controller suffix; null when the host shows no controller evidence, when no CI or two CIs carry that name, or when the CI is a load balancer.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>the hostname rules tried the whole label ("tx6dd630001-ilo") and found nothing, because no CI is named after the controller.</t>
-        </is>
-      </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
+          <t>the Linux Server CI "tx6dd630001", the label without "-ilo".</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>the hostname rules tried the whole label "tx6dd630001-ilo" and found nothing, because no CI is named after the controller.</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
           <t>hosts whose label ends with one of the controller suffixes, or whose OS text names a controller; both lists are declared in the script, at the top of the matching stage.</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>USEM Network Interface Name Match and USEM FQDN Name Hardware Match.</t>
         </is>
@@ -1067,27 +1261,43 @@
           <t>Network devices are scanned through their interface and VLAN addresses, and each of those carries a DNS label made of the device name plus an interface tail ("-cz04-hsrp-vlan705", "-atm1-v201", "-aom"), while the device CI is named with the leading part only. The rule walks the label from the longest prefix to the shortest and takes the first prefix that names exactly one network device.</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>sourceValue is the DNS field; the rule also reads the OS from sourcePayload.</t>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "1187423005",
+  "IP": "171.149.3.49",
+  "TRACKING_METHOD": "IP",
+  "OS": "Linux 2.6",
+  "DNS": "uspaltwrr01drm0119-cz04-hsrp-vlan705.network.bankofamerica.com"
+}</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
+          <t>sourceValue is the DNS field, "uspaltwrr01drm0119-cz04-hsrp-vlan705.network.bankofamerica.com"; the rule also reads the OS from sourcePayload.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
           <t>the sys_id of the one Network Gear or Load Balancer device CI named with a prefix of the label; null when the host shows no interface evidence, when no prefix names a device, or when a prefix names two.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>the hostname rules tried the whole label and USEM Management Interface Match looked for a controller suffix.</t>
-        </is>
-      </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
+          <t>the IP Switch CI "uspaltwrr01drm0119", the longest prefix of the label that names a device.</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>the hostname rules tried the whole label and USEM Management Interface Match looked for a controller suffix; "vlan705" is not one.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
           <t>hosts whose DNS domain is an interface domain (".network." in our feed) or whose label contains an interface marker segment such as "vlan705", "v201", "hsrp", "aom"; both lists are declared in the script, at the top of the matching stage.</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>USEM FQDN Name Hardware Match and USEM Load Balancer Service Match.</t>
         </is>
@@ -1112,27 +1322,44 @@
           <t>Some loads name the CI with the whole FQDN string instead of the short hostname (the appliance domains ending in .rpg are the usual case), so a short name search never finds them. This rule compares the complete scanned name with the name field, across the hardware tree.</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>sourceValue is the DNS field.</t>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "71973166",
+  "IP": "164.91.209.12",
+  "TRACKING_METHOD": "AGENT",
+  "OS": "Red Hat Enterprise Linux 8.10",
+  "DNS": "lva40bneehcs01.ecomm.devicenp.rpg",
+  "QG_HOSTID": "633781ed-019b-0002-2f2f-0050569d20ff"
+}</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
+          <t>sourceValue is the DNS field, "lva40bneehcs01.ecomm.devicenp.rpg".</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
           <t>the sys_id of the one hardware CI whose name is exactly the scanned FQDN; null when none or two carry it.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>every rule so far compared the short hostname or the fqdn field.</t>
-        </is>
-      </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
+          <t>the hardware CI named exactly "lva40bneehcs01.ecomm.devicenp.rpg", when it is the only one.</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>every rule so far compared the short hostname "lva40bneehcs01" or the fqdn field.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
           <t>CIs named with the full FQDN, which none of the earlier rules can see.</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>the IP address rules, and finally USEM FQDN Name Broad Match, the only rule allowed to search the whole CI table.</t>
         </is>
@@ -1157,27 +1384,43 @@
           <t>A virtual IP answered by a load balancer is not the balancer, and the hardware rules refuse the balancer device on purpose. Such hosts belong to the Load Balancer Service CI that models the VIP, and this rule finds it. It runs on the IP field so that VIPs without a DNS name are covered too.</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>sourceValue is the IP field; the rule also reads the OS and the DNS name from sourcePayload.</t>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "1202267231",
+  "IP": "171.203.142.26",
+  "TRACKING_METHOD": "IP",
+  "OS": "F5 Big IP",
+  "DNS": "crisp-tx.bankofamerica.com"
+}</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
+          <t>sourceValue is the IP field, "171.203.142.26"; the rule also reads the OS and the DNS name from sourcePayload.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
           <t>the sys_id of the one Load Balancer Service CI found by fqdn, then by name, then by address; null when the host shows no VIP evidence, when no service matches, or when two services carry the value.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>the hardware rules declined: a VIP has no serial, its name is not a server name, and the address belongs to a load balancer device.</t>
-        </is>
-      </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
+          <t>the Load Balancer Service CI "crisp-tx", whose fqdn is "crisp-tx.bankofamerica.com".</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>the hardware rules declined: a VIP has no serial, "crisp-tx" is not a server name, and the address belongs to a load balancer device.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
           <t>hosts with VIP evidence: an OS text naming a load balancer product, or a DNS label with a VIP marker segment such as "-vip" or "vs1"; both lists are declared in the script, at the top of the matching stage.</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>the IP address rules, for hosts that are not VIPs.</t>
         </is>
@@ -1202,27 +1445,42 @@
           <t>The first address rule. An address is the least trustworthy identifier we get: addresses move between machines and are shared by load balancers. It is used only for hosts without a serial and without a usable name, inside the class the scanned OS points at, and only when exactly one CI of that class carries it.</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>sourceValue is the IP field; the rule also reads the OS from sourcePayload.</t>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "83047621",
+  "IP": "30.162.178.21",
+  "TRACKING_METHOD": "IP",
+  "OS": "VMware ESXi 7.0.3 build 24723872"
+}</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
+          <t>sourceValue is the IP field, "30.162.178.21"; the rule also reads the OS from sourcePayload.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
           <t>the sys_id of the one CI of that class whose ip_address equals the scanned address; null when none or two carry it.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>all serial and name rules. A host without a DNS name makes every name rule decline.</t>
-        </is>
-      </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
+          <t>the ESX Server CI "vsdnesxm21", whose ip_address is "30.162.178.21"; a load balancer or a Windows CI on the same address is outside the class and cannot be picked.</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>all serial and name rules. The sample has no DNS name, so every name rule declined.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
           <t>DNS-less hosts, a small group in the feed, mostly ESXi management interfaces and appliances.</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>USEM IP Hardware Match searches the address across all hardware with extra safety checks; the adapter and layered address rules follow.</t>
         </is>
@@ -1247,27 +1505,42 @@
           <t>The address across the whole hardware tree, with two extra safety checks: the CI must not be a load balancer, and its class must not contradict the scanned OS.</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>sourceValue is the IP field; the rule also reads the OS from sourcePayload.</t>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "83047624",
+  "IP": "30.162.178.24",
+  "TRACKING_METHOD": "IP",
+  "OS": "Ubuntu / Tiny Core Linux / Linux 2.6.x / IBM ASM / HP StoreOnce / F5 Networks Big-IP / Cisco IOS Software"
+}</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
+          <t>sourceValue is the IP field, "30.162.178.24"; the rule also reads the OS from sourcePayload.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
           <t>the sys_id of the one hardware CI whose ip_address equals the scanned address, when it is not a load balancer and its class agrees with the scanned OS or is generic; null otherwise.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>USEM IP Class Match required the address to belong to one CI of the class the OS implies.</t>
-        </is>
-      </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
+          <t>the CI in the generic Server class whose ip_address is "30.162.178.24"; a Load Balancer on that address would be refused, and with a known OS a CI of a contradicting class would be too.</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>USEM IP Class Match required the address to belong to one CI of the class the OS implies; the sample OS is a list of guesses, so that rule declined without searching.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
           <t>DNS-less hosts whose CI is classed generically or whose OS gave no class.</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>USEM IP Adapter Match and USEM IP Layered Match.</t>
         </is>
@@ -1292,29 +1565,44 @@
           <t>Discovery stores one Network Adapter record per network card, and a multi-homed server keeps its addresses there rather than on the CI record. This rule finds the adapter carrying the scanned address and takes its owning CI.</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>sourceValue is the IP field.</t>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "83047622",
+  "IP": "30.162.178.22",
+  "TRACKING_METHOD": "IP",
+  "OS": "Ubuntu / Tiny Core Linux / Linux 2.6.x / IBM ASM / HP StoreOnce / F5 Networks Big-IP / Cisco IOS Software"
+}</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
+          <t>sourceValue is the IP field, "30.162.178.22".</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
           <t>the sys_id of the CI that owns the adapter carrying the scanned address; null when adapters of two different CIs carry it or the owner is a load balancer.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>the address rules so far looked at the ip_address field of the CI record itself.</t>
-        </is>
-      </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>hosts whose address is stored on an adapter record only.</t>
+          <t>the Server that owns the adapter "eth0" carrying "30.162.178.22"; the address is not written on the Server record itself.</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>USEM IP Layered Match and then the last-resort name rule.</t>
+          <t>the address rules so far read the ip_address field of the CI record, which holds nothing for the sample.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>hosts whose address is recorded on an adapter only.</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>USEM IP Layered Match and then the broad name rule.</t>
         </is>
       </c>
     </row>
@@ -1337,27 +1625,42 @@
           <t>Newer discovery writes each address as its own IP Address record linked to the adapter, and the adapter record itself may carry no address. This rule reads those records: IP Address -&gt; Network Adapter -&gt; CI.</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>sourceValue is the IP field.</t>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "83047623",
+  "IP": "30.162.178.23",
+  "TRACKING_METHOD": "IP",
+  "OS": "Ubuntu / Tiny Core Linux / Linux 2.6.x / IBM ASM / HP StoreOnce / F5 Networks Big-IP / Cisco IOS Software"
+}</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
+          <t>sourceValue is the IP field, "30.162.178.23".</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
           <t>the sys_id of the CI at the end of the chain IP Address -&gt; adapter -&gt; CI; null for several owners or a load balancer.</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>USEM IP Adapter Match looked for the address on the adapter records.</t>
-        </is>
-      </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
+          <t>the Server at the end of the chain IP Address "30.162.178.23" -&gt; adapter "eth0" -&gt; CI; neither the Server record nor the adapter record carries the address itself.</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>USEM IP Adapter Match looked for the address on the adapter records, which hold nothing for the sample.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
           <t>hosts whose address exists only as an IP Address record.</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>USEM FQDN Name Broad Match, and after that the out-of-box Qualys rules.</t>
         </is>
@@ -1382,34 +1685,50 @@
           <t>The one deliberately late, broad fallback: a CI named with the full FQDN anywhere in the CI table, classes outside the hardware tree included (a virtual machine instance, another logical CI). It still insists on a single owner outside the ignored classes.</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>sourceValue is the DNS field.</t>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "ID": "71973167",
+  "IP": "164.91.209.13",
+  "TRACKING_METHOD": "AGENT",
+  "OS": "Red Hat Enterprise Linux 8.10",
+  "DNS": "lva40bneehcs02.ecomm.devicenp.rpg"
+}</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
+          <t>sourceValue is the DNS field, "lva40bneehcs02.ecomm.devicenp.rpg".</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
           <t>the sys_id of the one CI in any class whose name is exactly the scanned FQDN; null when the name is shared.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>every hardware-scoped rule has declined for this host.</t>
-        </is>
-      </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
+          <t>the Virtual Machine Instance named "lva40bneehcs02.ecomm.devicenp.rpg", which lives outside the hardware tree and so escaped every earlier rule.</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>every hardware-scoped rule has declined for this host; USEM FQDN Name Hardware Match searched for the same name but only under Hardware.</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
           <t>the rare CI named with the full FQDN that lives outside the hardware tree.</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>the out-of-box Qualys rules (Qualys Host ID, Cloud Resource Id, FQDN, NetBIOS, DNS; the IP ones are inactive by default).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I20"/>
+  <autoFilter ref="A1:K20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1496,7 +1815,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>e.g. "wsaoi01zeapd1.sdi.corp.bankofamerica.com"</t>
+          <t>"wsaoi01zeapd1.sdi.corp.bankofamerica.com"</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1879,7 @@
       <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>The search below stays inside the class the OS points at (sub-classes included), so a Red Hat host can only land on a Linux Server and a Windows Server carrying the same value is never seen. "Windows Server 2016 Standard 64 bit Edition Version 1607" gives cmdb_ci_win_server (Windows Server). An unknown or multi-guess OS gives no class and the rule declines; the hardware-wide hostname match takes over. classFor() maps the OS text Qualys reports to the CMDB class the CI should be in, e.g. "Red Hat Enterprise Linux 9.8" is a Linux Server, "Windows Server 2016 Standard" a Windows Server and "VMware ESXi 7.0.3" an ESX Server. A string of guesses separated by "/" comes from an unauthenticated scan that could not identify the OS; three or more guesses give no class at all.</t>
+          <t>The search below stays inside the class the OS points at (sub-classes included), so a Red Hat host can only land on a Linux Server and a Windows Server carrying the same value is never seen. An unknown or multi-guess OS gives no class and the rule declines; the hardware-wide hostname match takes over. Sample: classFor("Windows Server 2016 Standard 64 bit Edition Version 1607") gives Windows Server, so pref is cmdb_ci_win_server and the search below runs on that class. classFor() maps the OS text Qualys reports to the CMDB class the CI should be in, e.g. "Red Hat Enterprise Linux 9.8" is a Linux Server, "Windows Server 2016 Standard" a Windows Server and "VMware ESXi 7.0.3" an ESX Server. A string of guesses separated by "/" comes from an unauthenticated scan that could not identify the OS; three or more guesses give no class at all.</t>
         </is>
       </c>
     </row>
@@ -1851,7 +2170,7 @@
       <c r="C26" s="4" t="inlineStr"/>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>With no domain to confirm, the class is the only safeguard against a namesake, and inside the class the name still has to be unique: two CIs with the same short name cannot be told apart here and the rule declines.</t>
+          <t>With no domain to confirm, the class is the only safeguard against a namesake, and inside the class the name still has to be unique: two CIs with the same short name cannot be told apart here and the rule declines. Sample: the search on cmdb_ci_win_server for name "wsaoi01zeapd1" finds the Windows Server "WSAOI01ZEAPD1" and no second row, so its sys_id is returned.</t>
         </is>
       </c>
     </row>
@@ -2106,7 +2425,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>e.g. "va2ausapabw0.bankofamerica.com"</t>
+          <t>"va2ausapabw0.bankofamerica.com"</t>
         </is>
       </c>
     </row>
@@ -2170,7 +2489,7 @@
       <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>This rule searches the whole hardware tree, so the class is not a filter here; it is checked at the end to reject a CI whose class contradicts the scan. "AIX 7.3 TL3" gives cmdb_ci_aix_server (AIX Server); an unknown OS gives no class and then no check is made. classFor() maps the OS text Qualys reports to the CMDB class the CI should be in, e.g. "Red Hat Enterprise Linux 9.8" is a Linux Server, "Windows Server 2016 Standard" a Windows Server and "VMware ESXi 7.0.3" an ESX Server. A string of guesses separated by "/" comes from an unauthenticated scan that could not identify the OS; three or more guesses give no class at all.</t>
+          <t>This rule searches the whole hardware tree, so the class is not a filter here; it is checked at the end to reject a CI whose class contradicts the scan. An unknown OS gives no class and then no check is made. Sample: classFor("AIX 7.3 TL3") gives AIX Server, so pref is cmdb_ci_aix_server; it is only used in the last stage. classFor() maps the OS text Qualys reports to the CMDB class the CI should be in, e.g. "Red Hat Enterprise Linux 9.8" is a Linux Server, "Windows Server 2016 Standard" a Windows Server and "VMware ESXi 7.0.3" an ESX Server. A string of guesses separated by "/" comes from an unauthenticated scan that could not identify the OS; three or more guesses give no class at all.</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2780,7 @@
       <c r="C26" s="4" t="inlineStr"/>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Nothing is filtered by class here; the two checks that follow provide the safety.</t>
+          <t>Nothing is filtered by class here; the two checks that follow provide the safety. Sample: the search on cmdb_ci_hardware for name "va2ausapabw0" finds the Server "va2ausapabw0", class cmdb_ci_server.</t>
         </is>
       </c>
     </row>
@@ -2524,7 +2843,7 @@
       <c r="C30" s="4" t="inlineStr"/>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>The first row is remembered with its class; a second row means two hardware CIs with one short name (a test and a production box, a retired and a rebuilt one), which the name alone cannot tell apart and the rule declines.</t>
+          <t>The first row is remembered with its class; a second row means two hardware CIs with one short name (a test and a production box, a retired and a rebuilt one), which the name alone cannot tell apart and the rule declines. Sample: one row, so id is the sys_id of "va2ausapabw0" and cls is "cmdb_ci_server". A second CI with that name would end the rule here.</t>
         </is>
       </c>
     </row>
@@ -2620,7 +2939,7 @@
       <c r="C36" s="4" t="inlineStr"/>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>When the OS gave a class, the CI found must sit inside it (sub-classes included) or be generically classed. A host that lands on a Windows Server by name or address is a namesake or a reused address, not the same machine, and its findings would go to the wrong owner.</t>
+          <t>When the OS gave a class, the CI found must sit inside it (sub-classes included) or be generically classed. A host that lands on a Windows Server by name or address is a namesake or a reused address, not the same machine, and its findings would go to the wrong owner. Sample: pref is cmdb_ci_aix_server; the CI is not an AIX Server, but cmdb_ci_server is in generic, so it passes and its sys_id is returned. A Windows Server named "va2ausapabw0" would fail both checks and the rule would decline.</t>
         </is>
       </c>
     </row>
@@ -2808,7 +3127,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>e.g. "tx6dd630001-ilo.bankofamerica.com"</t>
+          <t>"tx6dd630001-ilo.bankofamerica.com"</t>
         </is>
       </c>
     </row>
@@ -2840,7 +3159,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Position of the last hyphen; the controller suffix sits after it.</t>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -2873,7 +3192,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>The scanned OS text, lower-cased; empty when Qualys reported none.</t>
+          <t>"hp ilo"</t>
         </is>
       </c>
     </row>
@@ -2904,7 +3223,7 @@
       <c r="C10" s="4" t="inlineStr"/>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>The segment after the last hyphen is checked against the suffix list; when it is listed the server name is the label without it. Otherwise the OS text is checked for a controller word, and then the last segment is stripped whatever it is, because some controllers carry a site-specific tail instead ("crpchictx103-r" with OS "HP iLO"). Both habits are in the feed. Without either piece of evidence the host is not a controller and the rule must not touch it ("usposwks0042-x" with a Windows OS stays with the name rules). The label suffixes that mark a controller, and the words that name one in the OS text. Extend these two lists when a site uses another naming habit.</t>
+          <t>The segment after the last hyphen is checked against the suffix list; when it is listed the server name is the label without it. Otherwise the OS text is checked for a controller word, and then the last segment is stripped whatever it is, because some controllers carry a site-specific tail instead. Both habits are in the feed. Without either piece of evidence the host is not a controller and the rule must not touch it. Sample: the tail "ilo" is in suffixes, so base is "tx6dd630001". "crpchictx103-r" with OS "HP iLO" has an unlisted tail but a controller OS, so base would be "crpchictx103". "usposwks0042-x" with a Windows OS has neither, so the rule would decline. The label suffixes that mark a controller, and the words that name one in the OS text. Extend these two lists when a site uses another naming habit.</t>
         </is>
       </c>
     </row>
@@ -3082,7 +3401,7 @@
       <c r="C21" s="4" t="inlineStr"/>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>The controller can sit in front of a server, a storage node or a network device, so the whole hardware tree is searched. Two CIs with the server name cannot be told apart from the controller label alone and the rule declines; a load balancer is refused because a balancer answering on a management address is still not the scanned host.</t>
+          <t>The controller can sit in front of a server, a storage node or a network device, so the whole hardware tree is searched. Two CIs with the server name cannot be told apart from the controller label alone and the rule declines; a load balancer is refused because a balancer answering on a management address is still not the scanned host. Sample: the search on cmdb_ci_hardware for name "tx6dd630001" finds the Linux Server "tx6dd630001" and no second row; it is not a Load Balancer, so its sys_id is returned. Two servers named "crpchictx103" would make the rule decline.</t>
         </is>
       </c>
     </row>
@@ -3353,7 +3672,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>e.g. "uspaltwrr01drm0119-cz04-hsrp-vlan705.network.bankofamerica.com"</t>
+          <t>"uspaltwrr01drm0119-cz04-hsrp-vlan705.network.bankofamerica.com"</t>
         </is>
       </c>
     </row>
@@ -3369,7 +3688,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>The first label of the DNS name.</t>
+          <t>"uspaltwrr01drm0119-cz04-hsrp-vlan705"</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3899,7 @@
       <c r="C18" s="4" t="inlineStr"/>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>The rule goes on only when the DNS domain contains a listed interface domain or one of the segments after the first is a listed marker. Plenty of ordinary server names contain hyphens ("ah-1047132-001"); without this check the prefix walk would strip real hostnames and could land on an unrelated device. The domains under which devices are scanned per interface, and the label segments that mark an interface or VLAN address. Extend these two lists when a site uses another naming habit.</t>
+          <t>The rule goes on only when the DNS domain contains a listed interface domain or one of the segments after the first is a listed marker. Plenty of ordinary server names contain hyphens ("ah-1047132-001"); without this check the prefix walk would strip real hostnames and could land on an unrelated device. Sample: the name contains ".network." and the segment "vlan705" is the marker "vlan" followed by digits, so evidence is true on both counts. "ah-1047132-001.corp.bankofamerica.com" has neither and the rule would decline. The domains under which devices are scanned per interface, and the label segments that mark an interface or VLAN address. Extend these two lists when a site uses another naming habit.</t>
         </is>
       </c>
     </row>
@@ -3695,7 +4014,7 @@
       <c r="C25" s="4" t="inlineStr"/>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>One segment is dropped from the right at a time and the prefix is searched as a device name. The device name is the leading part of the label but its length varies by site, and trying the longest prefix first keeps "site-device-01" from being cut down to "site" when a CI with the longer name exists. The first prefix that finds anything decides: one CI is the match, two CIs mean the rule declines. Network devices live in two branches of the CMDB, Network Gear (switches, routers, firewalls) and Load Balancer, which the platform files under Server; both are searched and the hits are counted together.</t>
+          <t>One segment is dropped from the right at a time and the prefix is searched as a device name. The device name is the leading part of the label but its length varies by site, and trying the longest prefix first keeps "site-device-01" from being cut down to "site" when a CI with the longer name exists. The first prefix that finds anything decides: one CI is the match, two CIs mean the rule declines. Network devices live in two branches of the CMDB, Network Gear (switches, routers, firewalls) and Load Balancer, which the platform files under Server; both are searched and the hits are counted together. Sample: the prefixes tried are "uspaltwrr01drm0119-cz04-hsrp" (nothing), "uspaltwrr01drm0119-cz04" (nothing) and "uspaltwrr01drm0119", which names the IP Switch "uspaltwrr01drm0119" and nothing else, so its sys_id is returned. Two switches named "ustxrdnwl01rsm004z" would make the rule decline at that prefix.</t>
         </is>
       </c>
     </row>
@@ -4079,7 +4398,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>e.g. "lva40bneehcs01.ecomm.devicenp.rpg"</t>
+          <t>"lva40bneehcs01.ecomm.devicenp.rpg"</t>
         </is>
       </c>
     </row>
@@ -4127,7 +4446,7 @@
       <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>The name is compared with the whole string including the domain; the CI is accepted only when it is the single row.</t>
+          <t>The name is compared with the whole string including the domain; the CI is accepted only when it is the single row. Sample: the search on cmdb_ci_hardware for name "lva40bneehcs01.ecomm.devicenp.rpg" finds the Server named exactly that and no second row, so its sys_id is returned.</t>
         </is>
       </c>
     </row>
@@ -4365,7 +4684,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>e.g. "171.203.142.26"</t>
+          <t>"171.203.142.26"</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4717,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>e.g. "crisp-tx.bankofamerica.com", may be empty</t>
+          <t>"crisp-tx.bankofamerica.com", may be empty</t>
         </is>
       </c>
     </row>
@@ -4414,7 +4733,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>The first label of the DNS name, empty when there is no DNS name.</t>
+          <t>"crisp-tx"</t>
         </is>
       </c>
     </row>
@@ -4430,7 +4749,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>e.g. "f5 big ip"</t>
+          <t>"f5 big ip"</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4927,7 @@
       <c r="C19" s="4" t="inlineStr"/>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>The rule goes on only when the OS text contains a listed load balancer word or one of the label segments is a listed VIP marker. A Load Balancer Service must never be returned for an ordinary server that happens to share an address with a VIP; this check keeps the rule to the hosts that really are VIPs ("f5 big ip", "rbps-dev3-sve-vip"). The load balancer products looked for in the OS text, and the label segments that mark a virtual IP. Extend these two lists when a site uses another naming habit.</t>
+          <t>The rule goes on only when the OS text contains a listed load balancer word or one of the label segments is a listed VIP marker. A Load Balancer Service must never be returned for an ordinary server that happens to share an address with a VIP; this check keeps the rule to the hosts that really are VIPs. Sample: "f5 big ip" contains "f5", so evidence is true. "rbps-dev3-sve-vip.ecommnp.rpg" with OS "Linux 2.6" would qualify through the segment "vip"; "ah-1047132-001" with OS "Red Hat Enterprise Linux 9.8" has neither and the rule would decline. The load balancer products looked for in the OS text, and the label segments that mark a virtual IP. Extend these two lists when a site uses another naming habit.</t>
         </is>
       </c>
     </row>
@@ -4739,7 +5058,7 @@
       <c r="C27" s="4" t="inlineStr"/>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>The scanned DNS name is tried in the fqdn field, then in the name field, then the label in the name field, then the scanned address in ip_address. Each step accepts exactly one service; a step that finds two ends the rule with null, because a weaker piece of evidence could otherwise pick a different service; a step that finds nothing hands over to the next.</t>
+          <t>The scanned DNS name is tried in the fqdn field, then in the name field, then the label in the name field, then the scanned address in ip_address. Each step accepts exactly one service; a step that finds two ends the rule with null, because a weaker piece of evidence could otherwise pick a different service; a step that finds nothing hands over to the next. Sample: the first step, fqdn "crisp-tx.bankofamerica.com", finds the Load Balancer Service "crisp-tx" and no second row, so its sys_id is returned. A VIP without a DNS name and two services on "171.203.142.26" would reach the last step and decline there.</t>
         </is>
       </c>
     </row>
@@ -5157,7 +5476,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>e.g. "30.162.178.21"</t>
+          <t>"30.162.178.21"</t>
         </is>
       </c>
     </row>
@@ -5205,7 +5524,7 @@
       <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>The search below stays inside the class the OS points at (sub-classes included), so a Red Hat host can only land on a Linux Server and a Windows Server carrying the same value is never seen. "VMware ESXi 7.0.3 build 24723872" gives cmdb_ci_esx_server (ESX Server). An unknown or multi-guess OS gives no class and the rule declines; the hardware-wide address match takes over. classFor() maps the OS text Qualys reports to the CMDB class the CI should be in, e.g. "Red Hat Enterprise Linux 9.8" is a Linux Server, "Windows Server 2016 Standard" a Windows Server and "VMware ESXi 7.0.3" an ESX Server. A string of guesses separated by "/" comes from an unauthenticated scan that could not identify the OS; three or more guesses give no class at all.</t>
+          <t>The search below stays inside the class the OS points at (sub-classes included), so a Red Hat host can only land on a Linux Server and a Windows Server carrying the same value is never seen. An unknown or multi-guess OS gives no class and the rule declines; the hardware-wide address match takes over. Sample: classFor("VMware ESXi 7.0.3 build 24723872") gives ESX Server, so pref is cmdb_ci_esx_server and the search below runs on that class. classFor() maps the OS text Qualys reports to the CMDB class the CI should be in, e.g. "Red Hat Enterprise Linux 9.8" is a Linux Server, "Windows Server 2016 Standard" a Windows Server and "VMware ESXi 7.0.3" an ESX Server. A string of guesses separated by "/" comes from an unauthenticated scan that could not identify the OS; three or more guesses give no class at all.</t>
         </is>
       </c>
     </row>
@@ -5496,7 +5815,7 @@
       <c r="C25" s="4" t="inlineStr"/>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Inside the agreed class an address is reasonably safe: a virtual IP of a load balancer or a Windows machine that inherited the address sits outside the class and never appears. Two CIs of the class on one address (an address reused after a rebuild) still make the rule decline.</t>
+          <t>Inside the agreed class an address is reasonably safe: a virtual IP of a load balancer or a Windows machine that inherited the address sits outside the class and never appears. Two CIs of the class on one address (an address reused after a rebuild) still make the rule decline. Sample: the search on cmdb_ci_esx_server for ip_address "30.162.178.21" finds the ESX Server "vsdnesxm21" and no second row, so its sys_id is returned.</t>
         </is>
       </c>
     </row>
@@ -5751,7 +6070,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>e.g. "30.162.178.21"</t>
+          <t>"30.162.178.24"</t>
         </is>
       </c>
     </row>
@@ -5799,7 +6118,7 @@
       <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>This rule searches the whole hardware tree, so the class is not a filter here; it is checked at the end to reject a CI whose class contradicts the scan. "VMware ESXi 7.0.3 build 24723872" gives cmdb_ci_esx_server (ESX Server); an unknown OS gives no class and then no check is made. classFor() maps the OS text Qualys reports to the CMDB class the CI should be in, e.g. "Red Hat Enterprise Linux 9.8" is a Linux Server, "Windows Server 2016 Standard" a Windows Server and "VMware ESXi 7.0.3" an ESX Server. A string of guesses separated by "/" comes from an unauthenticated scan that could not identify the OS; three or more guesses give no class at all.</t>
+          <t>This rule searches the whole hardware tree, so the class is not a filter here; it is checked at the end to reject a CI whose class contradicts the scan. An unknown OS gives no class and then no check is made. Sample: classFor("Ubuntu / Tiny Core Linux / Linux 2.6.x / IBM ASM / HP StoreOnce / F5 Networks Big-IP / Cisco IOS Software") gives no class, so pref is ""; it is only used in the last stage. classFor() maps the OS text Qualys reports to the CMDB class the CI should be in, e.g. "Red Hat Enterprise Linux 9.8" is a Linux Server, "Windows Server 2016 Standard" a Windows Server and "VMware ESXi 7.0.3" an ESX Server. A string of guesses separated by "/" comes from an unauthenticated scan that could not identify the OS; three or more guesses give no class at all.</t>
         </is>
       </c>
     </row>
@@ -6154,7 +6473,7 @@
       <c r="C29" s="4" t="inlineStr"/>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Nothing is filtered by class here; the three checks that follow provide the safety.</t>
+          <t>Nothing is filtered by class here; the three checks that follow provide the safety. Sample: the search on cmdb_ci_hardware for ip_address "30.162.178.24" finds one CI in the generic Server class.</t>
         </is>
       </c>
     </row>
@@ -6217,7 +6536,7 @@
       <c r="C33" s="4" t="inlineStr"/>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>The first row is remembered with its class; a second row means an address answered by several CIs (a shared virtual IP, an address reused after a rebuild), which is never a safe match and the rule declines.</t>
+          <t>The first row is remembered with its class; a second row means an address answered by several CIs (a shared virtual IP, an address reused after a rebuild), which is never a safe match and the rule declines. Sample: one row, so id is the sys_id of that Server and cls is "cmdb_ci_server".</t>
         </is>
       </c>
     </row>
@@ -6313,7 +6632,7 @@
       <c r="C39" s="4" t="inlineStr"/>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>A scanned address that belongs to a load balancer is a virtual IP; the findings describe a pool member behind it, not the balancer.</t>
+          <t>A scanned address that belongs to a load balancer is a virtual IP; the findings describe a pool member behind it, not the balancer. Sample: the Server is not a Load Balancer, so the rule carries on. A Load Balancer on "30.162.178.24" would end it here.</t>
         </is>
       </c>
     </row>
@@ -6344,7 +6663,7 @@
       <c r="C41" s="4" t="inlineStr"/>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>When the OS gave a class, the CI found must sit inside it (sub-classes included) or be generically classed. A host that lands on a Windows Server by name or address is a namesake or a reused address, not the same machine, and its findings would go to the wrong owner.</t>
+          <t>When the OS gave a class, the CI found must sit inside it (sub-classes included) or be generically classed. A host that lands on a Windows Server by name or address is a namesake or a reused address, not the same machine, and its findings would go to the wrong owner. Sample: pref is empty for the sample, so no class check is made and the sys_id is returned. With OS "VMware ESXi 7.0.3", pref would be cmdb_ci_esx_server; the generic Server would still pass, a Windows Server would be rejected.</t>
         </is>
       </c>
     </row>
@@ -6532,7 +6851,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>e.g. "30.162.178.21"</t>
+          <t>"30.162.178.22"</t>
         </is>
       </c>
     </row>
@@ -6644,7 +6963,7 @@
       <c r="C11" s="4" t="inlineStr"/>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Adapters with the scanned address that belong to a CI outside the ignored classes.</t>
+          <t>Adapters with the scanned address that belong to a CI outside the ignored classes. Sample: the adapter "eth0" with ip_address "30.162.178.22" belongs to a Server; that is the one row the query returns.</t>
         </is>
       </c>
     </row>
@@ -6676,7 +6995,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Condition: the adapter carries the scanned address.</t>
+          <t>"30.162.178.22"</t>
         </is>
       </c>
     </row>
@@ -6739,7 +7058,7 @@
       <c r="C17" s="4" t="inlineStr"/>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Each distinct owning CI is counted once, so one server with two adapters on the address counts once and two servers count twice. Two different owners cannot be told apart by the address and the rule declines; a single owner that is a load balancer is refused too, because the address is then a virtual IP and the scanned host sits behind it.</t>
+          <t>Each distinct owning CI is counted once, so one server with two adapters on the address counts once and two servers count twice. Two different owners cannot be told apart by the address and the rule declines; a single owner that is a load balancer is refused too, because the address is then a virtual IP and the scanned host sits behind it. Sample: one adapter, one owner: count is 1, the owner is not a Load Balancer, so the sys_id of the Server is returned. A second server with an adapter on "30.162.178.22" would make the rule decline.</t>
         </is>
       </c>
     </row>
@@ -7040,7 +7359,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>e.g. "30.162.178.21"</t>
+          <t>"30.162.178.23"</t>
         </is>
       </c>
     </row>
@@ -7152,7 +7471,7 @@
       <c r="C11" s="4" t="inlineStr"/>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>nic.cmdb_ci reaches the CI two links away; the record must belong to an adapter that belongs to a CI outside the ignored classes.</t>
+          <t>nic.cmdb_ci reaches the CI two links away; the record must belong to an adapter that belongs to a CI outside the ignored classes. Sample: the IP Address record "30.162.178.23" belongs to the adapter "eth0", which belongs to a Server; that is the one row the query returns.</t>
         </is>
       </c>
     </row>
@@ -7201,7 +7520,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Condition: the IP Address record holds the scanned address.</t>
+          <t>"30.162.178.23"</t>
         </is>
       </c>
     </row>
@@ -7264,7 +7583,7 @@
       <c r="C18" s="4" t="inlineStr"/>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Each distinct owning CI is counted once, so one device with two address records counts once and two devices count twice. Two different owners cannot be told apart by the address and the rule declines; a single owner that is a load balancer is refused too, because the address is then a virtual IP and the scanned host sits behind it.</t>
+          <t>Each distinct owning CI is counted once, so one device with two address records counts once and two devices count twice. Two different owners cannot be told apart by the address and the rule declines; a single owner that is a load balancer is refused too, because the address is then a virtual IP and the scanned host sits behind it. Sample: one record, one owner: count is 1, the owner is not a Load Balancer, so the sys_id of the Server is returned.</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7884,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>e.g. "VMware-42 1a 9c 3f 7d 2e 61 b8-55 04 e2 91 6a 27 c3 08"</t>
+          <t>"VMware-42 1a 9c 3f 7d 2e 61 b8-55 04 e2 91 6a 27 c3 08"</t>
         </is>
       </c>
     </row>
@@ -7583,7 +7902,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Placeholder serials that vendors ship on thousands of machines ("To be filled by O.E.M.", "0123456789") would match dozens of CIs, so they are refused, as is anything shorter than four characters.</t>
+          <t>Placeholder serials that vendors ship on thousands of machines ("To be filled by O.E.M.", "0123456789") would match dozens of CIs, so they are refused, as is anything shorter than four characters. The sample serial is neither, so it goes through.</t>
         </is>
       </c>
     </row>
@@ -7631,7 +7950,7 @@
       <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>The search below stays inside the class the OS points at (sub-classes included), so a Red Hat host can only land on a Linux Server and a Windows Server carrying the same value is never seen. "Red Hat Enterprise Linux 9.8" gives cmdb_ci_linux_server (Linux Server). An unknown or multi-guess OS gives no class and the rule declines; the hardware-wide serial match takes over. classFor() maps the OS text Qualys reports to the CMDB class the CI should be in, e.g. "Red Hat Enterprise Linux 9.8" is a Linux Server, "Windows Server 2016 Standard" a Windows Server and "VMware ESXi 7.0.3" an ESX Server. A string of guesses separated by "/" comes from an unauthenticated scan that could not identify the OS; three or more guesses give no class at all.</t>
+          <t>The search below stays inside the class the OS points at (sub-classes included), so a Red Hat host can only land on a Linux Server and a Windows Server carrying the same value is never seen. An unknown or multi-guess OS gives no class and the rule declines; the hardware-wide serial match takes over. Sample: classFor("Red Hat Enterprise Linux 9.8") gives Linux Server, so pref is cmdb_ci_linux_server and the search below runs on that class. classFor() maps the OS text Qualys reports to the CMDB class the CI should be in, e.g. "Red Hat Enterprise Linux 9.8" is a Linux Server, "Windows Server 2016 Standard" a Windows Server and "VMware ESXi 7.0.3" an ESX Server. A string of guesses separated by "/" comes from an unauthenticated scan that could not identify the OS; three or more guesses give no class at all.</t>
         </is>
       </c>
     </row>
@@ -7922,7 +8241,7 @@
       <c r="C26" s="4" t="inlineStr"/>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Exact match on serial_number with the ignored classes left out. The CI is accepted only when it is the single row: two CIs sharing a serial do happen (a cloned virtual machine, a serial typed on the wrong record) and nothing here can tell them apart, so the rule declines and a later rule with different evidence gets its chance.</t>
+          <t>Exact match on serial_number with the ignored classes left out. The CI is accepted only when it is the single row: two CIs sharing a serial do happen (a cloned virtual machine, a serial typed on the wrong record) and nothing here can tell them apart, so the rule declines and a later rule with different evidence gets its chance. Sample: the search on cmdb_ci_linux_server for serial_number "VMware-42 1a 9c 3f 7d 2e 61 b8-55 04 e2 91 6a 27 c3 08" finds the Linux Server "ah-1047132-001" and no second row, so its sys_id is returned. A Windows Server with the same serial is outside the class and never appears.</t>
         </is>
       </c>
     </row>
@@ -8177,7 +8496,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>e.g. "lva40bneehcs01.ecomm.devicenp.rpg"</t>
+          <t>"lva40bneehcs02.ecomm.devicenp.rpg"</t>
         </is>
       </c>
     </row>
@@ -8225,7 +8544,7 @@
       <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>This is the only USEM rule that searches outside the hardware tree, which is why it runs last: every more precise rule has had its chance, and the ignore list still keeps the placeholder classes out.</t>
+          <t>This is the only USEM rule that searches outside the hardware tree, which is why it runs last: every more precise rule has had its chance, and the ignore list still keeps the placeholder classes out. Sample: the search on cmdb_ci for name "lva40bneehcs02.ecomm.devicenp.rpg" finds the Virtual Machine Instance named exactly that and no second row, so its sys_id is returned.</t>
         </is>
       </c>
     </row>
@@ -8463,7 +8782,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>e.g. "MXQ13005TC"</t>
+          <t>"MXQ13005TC"</t>
         </is>
       </c>
     </row>
@@ -8481,7 +8800,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Placeholder serials that vendors ship on thousands of machines ("To be filled by O.E.M.", "0123456789") would match dozens of CIs, so they are refused, as is anything shorter than four characters.</t>
+          <t>Placeholder serials that vendors ship on thousands of machines ("To be filled by O.E.M.", "0123456789") would match dozens of CIs, so they are refused, as is anything shorter than four characters. The sample serial is neither, so it goes through.</t>
         </is>
       </c>
     </row>
@@ -8529,7 +8848,7 @@
       <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>cmdb_ci_hardware is the parent of every device class, so nothing is filtered by class here; the safety is that the serial still has to belong to exactly one CI in the whole tree.</t>
+          <t>cmdb_ci_hardware is the parent of every device class, so nothing is filtered by class here; the safety is that the serial still has to belong to exactly one CI in the whole tree. Sample: the search on cmdb_ci_hardware for serial_number "MXQ13005TC" finds the Server "txr9gxcenah031" and no second row, so its sys_id is returned. A Storage Server loaded with the same serial would make the rule decline.</t>
         </is>
       </c>
     </row>
@@ -8765,7 +9084,7 @@
       <c r="C4" s="4" t="inlineStr"/>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>The first label of the DNS name must be exactly "sep" plus twelve hex characters; a server called "sepulveda01" must not be treated as a phone. The MAC is rebuilt in the four spellings the CMDB holds, because discovery tools and the call manager export write it differently ("64:F6:9D:D5:C9:B0", "64:f6:9d:d5:c9:b0", "64F69DD5C9B0", "64f69dd5c9b0").</t>
+          <t>The first label of the DNS name must be exactly "sep" plus twelve hex characters; a server called "sepulveda01" must not be treated as a phone. The MAC is rebuilt in the four spellings the CMDB holds, because discovery tools and the call manager export write it differently. Sample: "sep64f69dd5c9b0.voip.bankofamerica.com" gives the label "sep64f69dd5c9b0", the hex "64f69dd5c9b0" and candidates ["64:F6:9D:D5:C9:B0", "64:f6:9d:d5:c9:b0", "64F69DD5C9B0", "64f69dd5c9b0"].</t>
         </is>
       </c>
     </row>
@@ -8781,7 +9100,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>e.g. "sep64f69dd5c9b0"</t>
+          <t>"sep64f69dd5c9b0"</t>
         </is>
       </c>
     </row>
@@ -8863,7 +9182,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Cut the twelve characters into six pairs.</t>
+          <t>["64", "f6", "9d", "d5", "c9", "b0"]</t>
         </is>
       </c>
     </row>
@@ -8926,7 +9245,7 @@
       <c r="C14" s="4" t="inlineStr"/>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Three places are tried in turn: a network adapter with that MAC whose owner is an IP Phone CI (discovery usually stores the MAC on the adapter), the mac_address field on the phone record itself, and finally a phone named with the Unified CM device name ("SEP64F69DD5C9B0"). Each place must yield exactly one phone; two phones on one MAC or one device name is never guessed. Checking that the adapter owner really is an IP Phone is what keeps a switch or server adapter with a colliding MAC out.</t>
+          <t>Three places are tried in turn: a network adapter with that MAC whose owner is an IP Phone CI (discovery usually stores the MAC on the adapter), the mac_address field on the phone record itself, and finally a phone named with the Unified CM device name. Each place must yield exactly one phone; two phones on one MAC or one device name is never guessed. Checking that the adapter owner really is an IP Phone is what keeps a switch or server adapter with a colliding MAC out. Sample: the adapter "eth0" with mac_address "64:F6:9D:D5:C9:B0" belongs to the IP Phone "SEP64F69DD5C9B0"; count is 1, so that phone is returned from the first attempt. A phone with the MAC on its own record, or one simply named "SEP64F69DD5C9B0", would be found by the second or third attempt.</t>
         </is>
       </c>
     </row>
@@ -9330,7 +9649,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Condition: the phone is named with the SEP device name.</t>
+          <t>"SEP64F69DD5C9B0"</t>
         </is>
       </c>
     </row>
@@ -9536,7 +9855,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>e.g. "vsdnac22xsdi004.sdi.corp.bankofamerica.com"</t>
+          <t>"vsdnac22xsdi004.sdi.corp.bankofamerica.com"</t>
         </is>
       </c>
     </row>
@@ -9569,7 +9888,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>only used to break a tie</t>
+          <t>"30.206.199.36", only used to break a tie</t>
         </is>
       </c>
     </row>
@@ -9600,7 +9919,7 @@
       <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>The search below stays inside the class the OS points at (sub-classes included), so a Red Hat host can only land on a Linux Server and a Windows Server carrying the same value is never seen. "VMware ESXi 7.0.3 build 24723872" gives cmdb_ci_esx_server (ESX Server). An unknown or multi-guess OS gives no class and the rule declines; the hardware-wide FQDN match takes over. classFor() maps the OS text Qualys reports to the CMDB class the CI should be in, e.g. "Red Hat Enterprise Linux 9.8" is a Linux Server, "Windows Server 2016 Standard" a Windows Server and "VMware ESXi 7.0.3" an ESX Server. A string of guesses separated by "/" comes from an unauthenticated scan that could not identify the OS; three or more guesses give no class at all.</t>
+          <t>The search below stays inside the class the OS points at (sub-classes included), so a Red Hat host can only land on a Linux Server and a Windows Server carrying the same value is never seen. An unknown or multi-guess OS gives no class and the rule declines; the hardware-wide FQDN match takes over. Sample: classFor("VMware ESXi 7.0.3 build 24723872") gives ESX Server, so pref is cmdb_ci_esx_server and the search below runs on that class. classFor() maps the OS text Qualys reports to the CMDB class the CI should be in, e.g. "Red Hat Enterprise Linux 9.8" is a Linux Server, "Windows Server 2016 Standard" a Windows Server and "VMware ESXi 7.0.3" an ESX Server. A string of guesses separated by "/" comes from an unauthenticated scan that could not identify the OS; three or more guesses give no class at all.</t>
         </is>
       </c>
     </row>
@@ -9891,7 +10210,7 @@
       <c r="C26" s="4" t="inlineStr"/>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>pickFqdn() collects every CI of that class whose fqdn equals the scanned name and notes which of them also carry the scanned IP. One hit is the match. Duplicates do exist in the CMDB (a retired server and its rebuilt replacement, a cluster alias on two nodes); when exactly one of them carries the scanned IP that one is taken, otherwise the rule declines rather than guess.</t>
+          <t>pickFqdn() collects every CI of that class whose fqdn equals the scanned name and notes which of them also carry the scanned IP. One hit is the match. Duplicates do exist in the CMDB (a retired server and its rebuilt replacement, a cluster alias on two nodes); when exactly one of them carries the scanned IP that one is taken, otherwise the rule declines rather than guess. Sample: the ESX Server "vsdnac22xsdi004" has fqdn "vsdnac22xsdi004.sdi.corp.bankofamerica.com", so ids holds that one CI and its sys_id is returned. Were a second CI to carry the same fqdn, the one with ip_address "30.206.199.36" would be taken; if neither or both carried it, the rule would decline.</t>
         </is>
       </c>
     </row>
@@ -10275,7 +10594,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>e.g. "txr9gxcenah031.sdi.corp.bankofamerica.com"</t>
+          <t>"txr9gxcenah031.sdi.corp.bankofamerica.com"</t>
         </is>
       </c>
     </row>
@@ -10308,7 +10627,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>only used to break a tie</t>
+          <t>"171.135.28.125", only used to break a tie</t>
         </is>
       </c>
     </row>
@@ -10339,7 +10658,7 @@
       <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>pickFqdn() collects every CI under Hardware whose fqdn equals the scanned name and notes which of them also carry the scanned IP. One hit is the match. Duplicates do exist in the CMDB (a retired server and its rebuilt replacement, a cluster alias on two nodes); when exactly one of them carries the scanned IP that one is taken, otherwise the rule declines rather than guess.</t>
+          <t>pickFqdn() collects every CI under Hardware whose fqdn equals the scanned name and notes which of them also carry the scanned IP. One hit is the match. Duplicates do exist in the CMDB (a retired server and its rebuilt replacement, a cluster alias on two nodes); when exactly one of them carries the scanned IP that one is taken, otherwise the rule declines rather than guess. Sample: the Server "txr9gxcenah031" has fqdn "txr9gxcenah031.sdi.corp.bankofamerica.com", so ids holds that one CI and its sys_id is returned. Were a second CI to carry the same fqdn, the one with ip_address "171.135.28.125" would be taken; if neither or both carried it, the rule would decline.</t>
         </is>
       </c>
     </row>
@@ -10723,7 +11042,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>e.g. "ah-1047132-001.sdi.corp.bankofamerica.com"</t>
+          <t>"ah-1047132-001.sdi.corp.bankofamerica.com"</t>
         </is>
       </c>
     </row>
@@ -10804,7 +11123,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>only used to break a tie</t>
+          <t>"171.128.225.96", only used to break a tie</t>
         </is>
       </c>
     </row>
@@ -10835,7 +11154,7 @@
       <c r="C11" s="4" t="inlineStr"/>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>The search below stays inside the class the OS points at (sub-classes included), so a Red Hat host can only land on a Linux Server and a Windows Server carrying the same value is never seen. "Red Hat Enterprise Linux 9.8" gives cmdb_ci_linux_server (Linux Server). An unknown or multi-guess OS gives no class and the rule declines; the hardware-wide hostname-plus-domain match takes over. classFor() maps the OS text Qualys reports to the CMDB class the CI should be in, e.g. "Red Hat Enterprise Linux 9.8" is a Linux Server, "Windows Server 2016 Standard" a Windows Server and "VMware ESXi 7.0.3" an ESX Server. A string of guesses separated by "/" comes from an unauthenticated scan that could not identify the OS; three or more guesses give no class at all.</t>
+          <t>The search below stays inside the class the OS points at (sub-classes included), so a Red Hat host can only land on a Linux Server and a Windows Server carrying the same value is never seen. An unknown or multi-guess OS gives no class and the rule declines; the hardware-wide hostname-plus-domain match takes over. Sample: classFor("Red Hat Enterprise Linux 9.8") gives Linux Server, so pref is cmdb_ci_linux_server and the search below runs on that class. classFor() maps the OS text Qualys reports to the CMDB class the CI should be in, e.g. "Red Hat Enterprise Linux 9.8" is a Linux Server, "Windows Server 2016 Standard" a Windows Server and "VMware ESXi 7.0.3" an ESX Server. A string of guesses separated by "/" comes from an unauthenticated scan that could not identify the OS; three or more guesses give no class at all.</t>
         </is>
       </c>
     </row>
@@ -11126,7 +11445,7 @@
       <c r="C29" s="4" t="inlineStr"/>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>pickCombo() looks for CIs of that class named with the short hostname and keeps one only when its own record agrees with the scanned domain: fqdn equal to the scanned name, dns_domain equal to the scanned domain, or an fqdn that starts with the hostname and contains the domain. The same short name lives in several domains (a test and a production box both called app01), and this check is what keeps the findings off the namesake. One confirmed CI is the match; several with exactly one carrying the scanned IP gives that one; anything else declines.</t>
+          <t>pickCombo() looks for CIs of that class named with the short hostname and keeps one only when its own record agrees with the scanned domain: fqdn equal to the scanned name, dns_domain equal to the scanned domain, or an fqdn that starts with the hostname and contains the domain. The same short name lives in several domains (a test and a production box both called app01), and this check is what keeps the findings off the namesake. One confirmed CI is the match; several with exactly one carrying the scanned IP gives that one; anything else declines. Sample: the Linux Server is named "ah-1047132-001" and its dns_domain is "sdi.corp.bankofamerica.com", so it lands in good as the only entry and its sys_id is returned. A CI "ah-1047132-001" with dns_domain "lab.example.net" would be skipped; two confirmed CIs would be resolved by ip_address "171.128.225.96" or declined.</t>
         </is>
       </c>
     </row>
@@ -11575,7 +11894,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>e.g. "lrche01xtrapd01.sdi.corp.bankofamerica.com"</t>
+          <t>"lrche01xtrapd01.sdi.corp.bankofamerica.com"</t>
         </is>
       </c>
     </row>
@@ -11656,7 +11975,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>only used to break a tie</t>
+          <t>"171.128.140.192", only used to break a tie</t>
         </is>
       </c>
     </row>
@@ -11687,7 +12006,7 @@
       <c r="C11" s="4" t="inlineStr"/>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>pickCombo() looks for CIs under Hardware named with the short hostname and keeps one only when its own record agrees with the scanned domain: fqdn equal to the scanned name, dns_domain equal to the scanned domain, or an fqdn that starts with the hostname and contains the domain. The same short name lives in several domains (a test and a production box both called app01), and this check is what keeps the findings off the namesake. One confirmed CI is the match; several with exactly one carrying the scanned IP gives that one; anything else declines.</t>
+          <t>pickCombo() looks for CIs under Hardware named with the short hostname and keeps one only when its own record agrees with the scanned domain: fqdn equal to the scanned name, dns_domain equal to the scanned domain, or an fqdn that starts with the hostname and contains the domain. The same short name lives in several domains (a test and a production box both called app01), and this check is what keeps the findings off the namesake. One confirmed CI is the match; several with exactly one carrying the scanned IP gives that one; anything else declines. Sample: the Server is named "lrche01xtrapd01" and its dns_domain is "sdi.corp.bankofamerica.com", so it lands in good as the only entry and its sys_id is returned. A CI "lrche01xtrapd01" with dns_domain "lab.example.net" would be skipped; two confirmed CIs would be resolved by ip_address "171.128.140.192" or declined.</t>
         </is>
       </c>
     </row>
@@ -12136,7 +12455,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>e.g. "hklvteqoradbp3.hk.baml.com"</t>
+          <t>"hklvteqoradbp3.hk.baml.com"</t>
         </is>
       </c>
     </row>
@@ -12169,7 +12488,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>only used to break a tie</t>
+          <t>"167.202.60.26", only used to break a tie</t>
         </is>
       </c>
     </row>
@@ -12200,7 +12519,7 @@
       <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>cmdb_ip_address_dns_name ties one DNS Name record to one IP Address record; dot-walking reaches the rest: dns_name.name is the name on the DNS Name record and ip_address.nic.cmdb_ci is the CI owning the adapter that holds the address. Because the chain ends on whatever device holds the address, an alias resolves to the real machine.</t>
+          <t>cmdb_ip_address_dns_name ties one DNS Name record to one IP Address record; dot-walking reaches the rest: dns_name.name is the name on the DNS Name record and ip_address.nic.cmdb_ci is the CI owning the adapter that holds the address. Because the chain ends on whatever device holds the address, an alias resolves to the real machine. Sample: the DNS Name record "hklvteqoradbp3.hk.baml.com" is linked to the IP Address record "167.202.60.26", which belongs to the adapter "eth0" of the Linux Server "hklvteqoradbp3"; that is the one row the query returns.</t>
         </is>
       </c>
     </row>
@@ -12249,7 +12568,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Condition: the DNS Name record at the start of the chain is named with the scanned name.</t>
+          <t>"hklvteqoradbp3.hk.baml.com"</t>
         </is>
       </c>
     </row>
@@ -12312,7 +12631,7 @@
       <c r="C15" s="4" t="inlineStr"/>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Each distinct CI is counted once, and the CIs reached through the scanned address are noted. One CI is the match. A name that resolves to two devices (an alias moved between hosts, an old and a new record) is taken only when exactly one of them is reached through the scanned IP; otherwise the rule declines.</t>
+          <t>Each distinct CI is counted once, and the CIs reached through the scanned address are noted. One CI is the match. A name that resolves to two devices (an alias moved between hosts, an old and a new record) is taken only when exactly one of them is reached through the scanned IP; otherwise the rule declines. Sample: one row, so count is 1 and the sys_id of "hklvteqoradbp3" is returned. Were the name also linked to an address of a second device, ipOwners would hold only the CI reached through "167.202.60.26" and that one would be returned.</t>
         </is>
       </c>
     </row>

</xml_diff>